<commit_message>
Activate user-owned Around You image set
</commit_message>
<xml_diff>
--- a/assets-source/passenger/around-you/around-you-image-inventory.xlsx
+++ b/assets-source/passenger/around-you/around-you-image-inventory.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0bb277b4b6a7404c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="R6ff28046eebc41e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6e2087d121824cae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="Ra249ea74218041df"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -608,7 +608,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="27" t="str">
-        <x:v>P1.2 assisted image sourcing · 100 places across the STREEX corridor</x:v>
+        <x:v>P1.3 user-photo activation · 100 places across the STREEX corridor</x:v>
       </x:c>
       <x:c r="B2" s="27"/>
       <x:c r="C2" s="27"/>
@@ -647,7 +647,7 @@
         <x:v>Original upload folder</x:v>
       </x:c>
       <x:c r="B5" s="30" t="str">
-        <x:v>assets-source/passenger/around-you/</x:v>
+        <x:v>assets-source/passenger/around-you/user-originals/</x:v>
       </x:c>
       <x:c r="C5" s="28"/>
       <x:c r="D5" s="28"/>
@@ -686,10 +686,10 @@
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
       <x:c r="A8" s="29" t="str">
-        <x:v>Rights rule</x:v>
+        <x:v>Privacy rule</x:v>
       </x:c>
       <x:c r="B8" s="30" t="str">
-        <x:v>Fill source/author and license/permission before an image is enabled in the app.</x:v>
+        <x:v>Strip EXIF/GPS from public copies; keep raw originals local and ignored.</x:v>
       </x:c>
       <x:c r="C8" s="28"/>
       <x:c r="D8" s="28"/>
@@ -773,7 +773,7 @@
       </x:c>
       <x:c r="B14" s="33" t="n">
         <x:f>COUNTIF('Inventory'!I5:I104,"Own local asset")</x:f>
-        <x:v>6</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C14" s="28"/>
       <x:c r="D14" s="28"/>
@@ -788,7 +788,7 @@
       </x:c>
       <x:c r="B15" s="33" t="n">
         <x:f>COUNTIF('Inventory'!I5:I104,"Original staged — rights recorded")</x:f>
-        <x:v>15</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C15" s="28"/>
       <x:c r="D15" s="28"/>
@@ -803,7 +803,7 @@
       </x:c>
       <x:c r="B16" s="33" t="n">
         <x:f>COUNTIF('Inventory'!I5:I104,"Shared fallback")</x:f>
-        <x:v>11</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="28"/>
@@ -833,7 +833,7 @@
       </x:c>
       <x:c r="B18" s="33" t="n">
         <x:f>COUNTIF('Inventory'!J5:J104,"Yes")</x:f>
-        <x:v>79</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C18" s="28"/>
       <x:c r="D18" s="28"/>
@@ -1099,7 +1099,7 @@
         <x:v>salt-lake-valley.jpg</x:v>
       </x:c>
       <x:c r="H5" s="72" t="str">
-        <x:v>/images/passenger/around-you/salt-lake-valley.webp</x:v>
+        <x:v>/images/passenger/around-you/user/salt-lake-valley-juan.webp</x:v>
       </x:c>
       <x:c r="I5" s="74" t="str">
         <x:v>Own local asset</x:v>
@@ -1116,13 +1116,15 @@
       <x:c r="M5" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N5" s="72" t="str">
-        <x:v>https://www.visitsaltlake.com/</x:v>
-      </x:c>
-      <x:c r="O5" s="72" t="str"/>
-      <x:c r="P5" s="72" t="str"/>
+      <x:c r="N5" s="72" t="str"/>
+      <x:c r="O5" s="72" t="str">
+        <x:v>STREEX-owned original — Juan</x:v>
+      </x:c>
+      <x:c r="P5" s="72" t="str">
+        <x:v>User-owned original; permission confirmed</x:v>
+      </x:c>
       <x:c r="Q5" s="72" t="str">
-        <x:v>Current optimized asset is available; replace only if a stronger original is supplied.</x:v>
+        <x:v>Selected from IMG_3418.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
@@ -1148,7 +1150,7 @@
         <x:v>wasatch-back.jpg</x:v>
       </x:c>
       <x:c r="H6" s="76" t="str">
-        <x:v>/images/passenger/around-you/wasatch-back.webp</x:v>
+        <x:v>/images/passenger/around-you/user/wasatch-back-juan.webp</x:v>
       </x:c>
       <x:c r="I6" s="74" t="str">
         <x:v>Own local asset</x:v>
@@ -1165,13 +1167,15 @@
       <x:c r="M6" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N6" s="76" t="str">
-        <x:v>https://www.visitparkcity.com/</x:v>
-      </x:c>
-      <x:c r="O6" s="76" t="str"/>
-      <x:c r="P6" s="76" t="str"/>
+      <x:c r="N6" s="76" t="str"/>
+      <x:c r="O6" s="76" t="str">
+        <x:v>STREEX-owned original — Juan</x:v>
+      </x:c>
+      <x:c r="P6" s="76" t="str">
+        <x:v>User-owned original; permission confirmed</x:v>
+      </x:c>
       <x:c r="Q6" s="76" t="str">
-        <x:v>Current optimized asset is available; replace only if a stronger original is supplied.</x:v>
+        <x:v>Selected from IMG_0338.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -1197,7 +1201,7 @@
         <x:v>downtown-salt-lake-city.jpg</x:v>
       </x:c>
       <x:c r="H7" s="72" t="str">
-        <x:v>/images/passenger/around-you/downtown-slc.jpg</x:v>
+        <x:v>/images/passenger/around-you/user/downtown-salt-lake-city-juan.webp</x:v>
       </x:c>
       <x:c r="I7" s="74" t="str">
         <x:v>Own local asset</x:v>
@@ -1214,13 +1218,15 @@
       <x:c r="M7" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N7" s="72" t="str">
-        <x:v>https://www.slc.gov/</x:v>
-      </x:c>
-      <x:c r="O7" s="72" t="str"/>
-      <x:c r="P7" s="72" t="str"/>
+      <x:c r="N7" s="72" t="str"/>
+      <x:c r="O7" s="72" t="str">
+        <x:v>STREEX-owned original — Juan</x:v>
+      </x:c>
+      <x:c r="P7" s="72" t="str">
+        <x:v>User-owned original; permission confirmed</x:v>
+      </x:c>
       <x:c r="Q7" s="72" t="str">
-        <x:v>Current optimized asset is available; replace only if a stronger original is supplied.</x:v>
+        <x:v>Selected from IMG_0659.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
@@ -1245,9 +1251,11 @@
       <x:c r="G8" s="76" t="str">
         <x:v>utah-state-capitol.jpg</x:v>
       </x:c>
-      <x:c r="H8" s="76" t="str"/>
-      <x:c r="I8" s="77" t="str">
-        <x:v>Original staged — rights recorded</x:v>
+      <x:c r="H8" s="76" t="str">
+        <x:v>/images/passenger/around-you/user/utah-state-capitol-juan.webp</x:v>
+      </x:c>
+      <x:c r="I8" s="74" t="str">
+        <x:v>Own local asset</x:v>
       </x:c>
       <x:c r="J8" s="75" t="str">
         <x:v>No</x:v>
@@ -1261,17 +1269,15 @@
       <x:c r="M8" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N8" s="76" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:Utah_State_Capitol_UT1.jpg</x:v>
-      </x:c>
+      <x:c r="N8" s="76" t="str"/>
       <x:c r="O8" s="76" t="str">
-        <x:v>Wikimedia Commons — Acroterion</x:v>
+        <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
       <x:c r="P8" s="76" t="str">
-        <x:v>CC BY-SA 4.0 — attribution and share-alike required</x:v>
+        <x:v>User-owned original; permission confirmed</x:v>
       </x:c>
       <x:c r="Q8" s="76" t="str">
-        <x:v>Original staged in assets-source/passenger/around-you; rights recorded. Optimize/crop to public WebP in P1.3. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Selected from IMG_0244.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -1296,9 +1302,11 @@
       <x:c r="G9" s="72" t="str">
         <x:v>temple-square.jpg</x:v>
       </x:c>
-      <x:c r="H9" s="72" t="str"/>
-      <x:c r="I9" s="77" t="str">
-        <x:v>Original staged — rights recorded</x:v>
+      <x:c r="H9" s="72" t="str">
+        <x:v>/images/passenger/around-you/user/temple-square-juan.webp</x:v>
+      </x:c>
+      <x:c r="I9" s="74" t="str">
+        <x:v>Own local asset</x:v>
       </x:c>
       <x:c r="J9" s="75" t="str">
         <x:v>No</x:v>
@@ -1312,17 +1320,15 @@
       <x:c r="M9" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N9" s="72" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:2013_Temple_Square_Salt_Lake_City_(3).jpg</x:v>
-      </x:c>
+      <x:c r="N9" s="72" t="str"/>
       <x:c r="O9" s="72" t="str">
-        <x:v>Wikimedia Commons — Chris06</x:v>
+        <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
       <x:c r="P9" s="72" t="str">
-        <x:v>CC BY-SA 4.0 — attribution and share-alike required</x:v>
+        <x:v>User-owned original; permission confirmed</x:v>
       </x:c>
       <x:c r="Q9" s="72" t="str">
-        <x:v>Original staged in assets-source/passenger/around-you; rights recorded. Optimize/crop to public WebP in P1.3. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Selected from IMG_0335.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
@@ -1347,9 +1353,11 @@
       <x:c r="G10" s="76" t="str">
         <x:v>city-creek-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H10" s="76" t="str"/>
-      <x:c r="I10" s="77" t="str">
-        <x:v>Original staged — rights recorded</x:v>
+      <x:c r="H10" s="76" t="str">
+        <x:v>/images/passenger/around-you/user/city-creek-canyon-juan.webp</x:v>
+      </x:c>
+      <x:c r="I10" s="74" t="str">
+        <x:v>Own local asset</x:v>
       </x:c>
       <x:c r="J10" s="75" t="str">
         <x:v>No</x:v>
@@ -1363,17 +1371,15 @@
       <x:c r="M10" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N10" s="76" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:Ensign_Peak_above_City_Creek_Canyon_-_Salt_Lake_City,_Utah_-_8_June_2024.jpg</x:v>
-      </x:c>
+      <x:c r="N10" s="76" t="str"/>
       <x:c r="O10" s="76" t="str">
-        <x:v>Wikimedia Commons — Beneathtimp</x:v>
+        <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
       <x:c r="P10" s="76" t="str">
-        <x:v>CC0 — no attribution required; attribution retained in inventory</x:v>
+        <x:v>User-owned original; permission confirmed</x:v>
       </x:c>
       <x:c r="Q10" s="76" t="str">
-        <x:v>Original staged in assets-source/passenger/around-you; rights recorded. Optimize/crop to public WebP in P1.3. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Selected from IMG_0976.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
@@ -1398,9 +1404,11 @@
       <x:c r="G11" s="72" t="str">
         <x:v>liberty-park.jpg</x:v>
       </x:c>
-      <x:c r="H11" s="72" t="str"/>
-      <x:c r="I11" s="77" t="str">
-        <x:v>Original staged — rights recorded</x:v>
+      <x:c r="H11" s="72" t="str">
+        <x:v>/images/passenger/around-you/user/liberty-park-juan.webp</x:v>
+      </x:c>
+      <x:c r="I11" s="74" t="str">
+        <x:v>Own local asset</x:v>
       </x:c>
       <x:c r="J11" s="75" t="str">
         <x:v>No</x:v>
@@ -1414,17 +1422,15 @@
       <x:c r="M11" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N11" s="72" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:Liberty_Park,_Salt_Lake_City,_UT.jpg</x:v>
-      </x:c>
+      <x:c r="N11" s="72" t="str"/>
       <x:c r="O11" s="72" t="str">
-        <x:v>Wikimedia Commons — Pollardjosephd</x:v>
+        <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
       <x:c r="P11" s="72" t="str">
-        <x:v>CC BY-SA 4.0 — attribution and share-alike required</x:v>
+        <x:v>User-owned original; permission confirmed</x:v>
       </x:c>
       <x:c r="Q11" s="72" t="str">
-        <x:v>Original staged in assets-source/passenger/around-you; rights recorded. Optimize/crop to public WebP in P1.3. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Selected from IMG_8789.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
@@ -1654,7 +1660,7 @@
         <x:v>great-salt-lake.jpg</x:v>
       </x:c>
       <x:c r="H16" s="76" t="str">
-        <x:v>/images/passenger/around-you/great-salt-lake.jpg</x:v>
+        <x:v>/images/passenger/around-you/user/great-salt-lake-juan.webp</x:v>
       </x:c>
       <x:c r="I16" s="74" t="str">
         <x:v>Own local asset</x:v>
@@ -1671,13 +1677,15 @@
       <x:c r="M16" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N16" s="76" t="str">
-        <x:v>https://stateparks.utah.gov/parks/great-salt-lake/</x:v>
-      </x:c>
-      <x:c r="O16" s="76" t="str"/>
-      <x:c r="P16" s="76" t="str"/>
+      <x:c r="N16" s="76" t="str"/>
+      <x:c r="O16" s="76" t="str">
+        <x:v>STREEX-owned original — Juan</x:v>
+      </x:c>
+      <x:c r="P16" s="76" t="str">
+        <x:v>User-owned original; permission confirmed</x:v>
+      </x:c>
       <x:c r="Q16" s="76" t="str">
-        <x:v>Current optimized asset is available; replace only if a stronger original is supplied.</x:v>
+        <x:v>Selected from IMG_6450.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
@@ -1753,9 +1761,11 @@
       <x:c r="G18" s="76" t="str">
         <x:v>lagoon-amusement-park.jpg</x:v>
       </x:c>
-      <x:c r="H18" s="76" t="str"/>
-      <x:c r="I18" s="77" t="str">
-        <x:v>Original staged — rights recorded</x:v>
+      <x:c r="H18" s="76" t="str">
+        <x:v>/images/passenger/around-you/user/lagoon-amusement-park-juan.webp</x:v>
+      </x:c>
+      <x:c r="I18" s="74" t="str">
+        <x:v>Own local asset</x:v>
       </x:c>
       <x:c r="J18" s="75" t="str">
         <x:v>No</x:v>
@@ -1769,17 +1779,15 @@
       <x:c r="M18" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N18" s="76" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:Lagoon_carousel.JPG</x:v>
-      </x:c>
+      <x:c r="N18" s="76" t="str"/>
       <x:c r="O18" s="76" t="str">
-        <x:v>Wikimedia Commons — Davehi1</x:v>
+        <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
       <x:c r="P18" s="76" t="str">
-        <x:v>Public domain</x:v>
+        <x:v>User-owned original; permission confirmed</x:v>
       </x:c>
       <x:c r="Q18" s="76" t="str">
-        <x:v>Original staged in assets-source/passenger/around-you; rights recorded. Optimize/crop to public WebP in P1.3. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Selected from IMG_2568.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
@@ -1855,9 +1863,11 @@
       <x:c r="G20" s="76" t="str">
         <x:v>antelope-island.jpg</x:v>
       </x:c>
-      <x:c r="H20" s="76" t="str"/>
-      <x:c r="I20" s="77" t="str">
-        <x:v>Original staged — rights recorded</x:v>
+      <x:c r="H20" s="76" t="str">
+        <x:v>/images/passenger/around-you/user/antelope-island-juan.webp</x:v>
+      </x:c>
+      <x:c r="I20" s="74" t="str">
+        <x:v>Own local asset</x:v>
       </x:c>
       <x:c r="J20" s="75" t="str">
         <x:v>No</x:v>
@@ -1871,17 +1881,15 @@
       <x:c r="M20" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N20" s="76" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:Sunset_on_Antelope_Island,_Utah.jpg</x:v>
-      </x:c>
+      <x:c r="N20" s="76" t="str"/>
       <x:c r="O20" s="76" t="str">
-        <x:v>Wikimedia Commons — Shaun Fisher</x:v>
+        <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
       <x:c r="P20" s="76" t="str">
-        <x:v>CC BY 2.0 — attribution required</x:v>
+        <x:v>User-owned original; permission confirmed</x:v>
       </x:c>
       <x:c r="Q20" s="76" t="str">
-        <x:v>Original staged in assets-source/passenger/around-you; rights recorded. Optimize/crop to public WebP in P1.3. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Selected from IMG_6483.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
@@ -1907,7 +1915,7 @@
         <x:v>park-city.jpg</x:v>
       </x:c>
       <x:c r="H21" s="72" t="str">
-        <x:v>/images/passenger/around-you/park-city.jpg</x:v>
+        <x:v>/images/passenger/around-you/user/park-city-juan.webp</x:v>
       </x:c>
       <x:c r="I21" s="74" t="str">
         <x:v>Own local asset</x:v>
@@ -1924,13 +1932,15 @@
       <x:c r="M21" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N21" s="72" t="str">
-        <x:v>https://www.visitparkcity.com/things-to-do/museums-history/park-city-history/</x:v>
-      </x:c>
-      <x:c r="O21" s="72" t="str"/>
-      <x:c r="P21" s="72" t="str"/>
+      <x:c r="N21" s="72" t="str"/>
+      <x:c r="O21" s="72" t="str">
+        <x:v>STREEX-owned original — Juan</x:v>
+      </x:c>
+      <x:c r="P21" s="72" t="str">
+        <x:v>User-owned original; permission confirmed</x:v>
+      </x:c>
       <x:c r="Q21" s="72" t="str">
-        <x:v>Current optimized asset is available; replace only if a stronger original is supplied.</x:v>
+        <x:v>Selected from IMG_4516.JPG; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
@@ -1955,9 +1965,11 @@
       <x:c r="G22" s="76" t="str">
         <x:v>historic-main-street.jpg</x:v>
       </x:c>
-      <x:c r="H22" s="76" t="str"/>
-      <x:c r="I22" s="77" t="str">
-        <x:v>Original staged — rights recorded</x:v>
+      <x:c r="H22" s="76" t="str">
+        <x:v>/images/passenger/around-you/user/historic-main-street-juan.webp</x:v>
+      </x:c>
+      <x:c r="I22" s="74" t="str">
+        <x:v>Own local asset</x:v>
       </x:c>
       <x:c r="J22" s="75" t="str">
         <x:v>No</x:v>
@@ -1971,17 +1983,15 @@
       <x:c r="M22" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N22" s="76" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:Main_Street_Park_City_Utah.JPG</x:v>
-      </x:c>
+      <x:c r="N22" s="76" t="str"/>
       <x:c r="O22" s="76" t="str">
-        <x:v>Wikimedia Commons — Mrs keyser soze</x:v>
+        <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
       <x:c r="P22" s="76" t="str">
-        <x:v>CC BY-SA 3.0 — attribution and share-alike required</x:v>
+        <x:v>User-owned original; permission confirmed</x:v>
       </x:c>
       <x:c r="Q22" s="76" t="str">
-        <x:v>Original staged in assets-source/passenger/around-you; rights recorded. Optimize/crop to public WebP in P1.3. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Selected from IMG_8782.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
@@ -2007,7 +2017,7 @@
         <x:v>utah-olympic-park.jpg</x:v>
       </x:c>
       <x:c r="H23" s="72" t="str">
-        <x:v>/images/passenger/around-you/utah-olympic-park.jpg</x:v>
+        <x:v>/images/passenger/around-you/user/utah-olympic-park-juan.webp</x:v>
       </x:c>
       <x:c r="I23" s="74" t="str">
         <x:v>Own local asset</x:v>
@@ -2024,13 +2034,15 @@
       <x:c r="M23" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N23" s="72" t="str">
-        <x:v>https://www.visitparkcity.com/things-to-do/utah-olympic-park/</x:v>
-      </x:c>
-      <x:c r="O23" s="72" t="str"/>
-      <x:c r="P23" s="72" t="str"/>
+      <x:c r="N23" s="72" t="str"/>
+      <x:c r="O23" s="72" t="str">
+        <x:v>STREEX-owned original — Juan</x:v>
+      </x:c>
+      <x:c r="P23" s="72" t="str">
+        <x:v>User-owned original; permission confirmed</x:v>
+      </x:c>
       <x:c r="Q23" s="72" t="str">
-        <x:v>Current optimized asset is available; replace only if a stronger original is supplied.</x:v>
+        <x:v>Selected from IMG_1099.JPG; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
@@ -2055,9 +2067,11 @@
       <x:c r="G24" s="76" t="str">
         <x:v>kimball-junction.jpg</x:v>
       </x:c>
-      <x:c r="H24" s="76" t="str"/>
-      <x:c r="I24" s="77" t="str">
-        <x:v>Original staged — rights recorded</x:v>
+      <x:c r="H24" s="76" t="str">
+        <x:v>/images/passenger/around-you/user/kimball-junction-juan.webp</x:v>
+      </x:c>
+      <x:c r="I24" s="74" t="str">
+        <x:v>Own local asset</x:v>
       </x:c>
       <x:c r="J24" s="75" t="str">
         <x:v>No</x:v>
@@ -2071,17 +2085,15 @@
       <x:c r="M24" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N24" s="76" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:Kimball_Junction_PC_to_SLC_connector.jpg</x:v>
-      </x:c>
+      <x:c r="N24" s="76" t="str"/>
       <x:c r="O24" s="76" t="str">
-        <x:v>Wikimedia Commons — Eyezak mad</x:v>
+        <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
       <x:c r="P24" s="76" t="str">
-        <x:v>CC BY 4.0 — attribution required</x:v>
+        <x:v>User-owned original; permission confirmed</x:v>
       </x:c>
       <x:c r="Q24" s="76" t="str">
-        <x:v>Original staged in assets-source/passenger/around-you; rights recorded. Optimize/crop to public WebP in P1.3. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Selected from IMG_4721.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
@@ -2106,9 +2118,11 @@
       <x:c r="G25" s="72" t="str">
         <x:v>deer-valley.jpg</x:v>
       </x:c>
-      <x:c r="H25" s="72" t="str"/>
-      <x:c r="I25" s="77" t="str">
-        <x:v>Original staged — rights recorded</x:v>
+      <x:c r="H25" s="72" t="str">
+        <x:v>/images/passenger/around-you/user/deer-valley-juan.webp</x:v>
+      </x:c>
+      <x:c r="I25" s="74" t="str">
+        <x:v>Own local asset</x:v>
       </x:c>
       <x:c r="J25" s="75" t="str">
         <x:v>No</x:v>
@@ -2122,17 +2136,15 @@
       <x:c r="M25" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N25" s="72" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:Deer_Valley._Utah.jpg</x:v>
-      </x:c>
+      <x:c r="N25" s="72" t="str"/>
       <x:c r="O25" s="72" t="str">
-        <x:v>Wikimedia Commons — Tiraspolsky</x:v>
+        <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
       <x:c r="P25" s="72" t="str">
-        <x:v>CC BY-SA 4.0 — attribution and share-alike required</x:v>
+        <x:v>User-owned original; permission confirmed</x:v>
       </x:c>
       <x:c r="Q25" s="72" t="str">
-        <x:v>Original staged in assets-source/passenger/around-you; rights recorded. Optimize/crop to public WebP in P1.3. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Selected from IMG_0967.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
@@ -2354,13 +2366,13 @@
         <x:v>the-gateway.jpg</x:v>
       </x:c>
       <x:c r="H30" s="76" t="str">
-        <x:v>/images/passenger/around-you/downtown-slc.jpg</x:v>
-      </x:c>
-      <x:c r="I30" s="78" t="str">
-        <x:v>Shared fallback</x:v>
-      </x:c>
-      <x:c r="J30" s="79" t="str">
-        <x:v>Yes</x:v>
+        <x:v>/images/passenger/around-you/user/the-gateway-juan.webp</x:v>
+      </x:c>
+      <x:c r="I30" s="74" t="str">
+        <x:v>Own local asset</x:v>
+      </x:c>
+      <x:c r="J30" s="75" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K30" s="76" t="n">
         <x:v>1</x:v>
@@ -2371,13 +2383,15 @@
       <x:c r="M30" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N30" s="76" t="str">
-        <x:v>https://atthegateway.com/</x:v>
-      </x:c>
-      <x:c r="O30" s="76" t="str"/>
-      <x:c r="P30" s="76" t="str"/>
+      <x:c r="N30" s="76" t="str"/>
+      <x:c r="O30" s="76" t="str">
+        <x:v>STREEX-owned original — Juan</x:v>
+      </x:c>
+      <x:c r="P30" s="76" t="str">
+        <x:v>User-owned original; permission confirmed</x:v>
+      </x:c>
       <x:c r="Q30" s="76" t="str">
-        <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Selected from IMG_1412.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
@@ -2452,13 +2466,13 @@
         <x:v>swaner-preserve.jpg</x:v>
       </x:c>
       <x:c r="H32" s="76" t="str">
-        <x:v>/images/passenger/around-you/wasatch-back.webp</x:v>
-      </x:c>
-      <x:c r="I32" s="78" t="str">
-        <x:v>Shared fallback</x:v>
-      </x:c>
-      <x:c r="J32" s="79" t="str">
-        <x:v>Yes</x:v>
+        <x:v>/images/passenger/around-you/user/swaner-preserve-juan.webp</x:v>
+      </x:c>
+      <x:c r="I32" s="74" t="str">
+        <x:v>Own local asset</x:v>
+      </x:c>
+      <x:c r="J32" s="75" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K32" s="76" t="n">
         <x:v>1</x:v>
@@ -2469,13 +2483,15 @@
       <x:c r="M32" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N32" s="76" t="str">
-        <x:v>https://swanerecocenter.org/</x:v>
-      </x:c>
-      <x:c r="O32" s="76" t="str"/>
-      <x:c r="P32" s="76" t="str"/>
+      <x:c r="N32" s="76" t="str"/>
+      <x:c r="O32" s="76" t="str">
+        <x:v>STREEX-owned original — Juan</x:v>
+      </x:c>
+      <x:c r="P32" s="76" t="str">
+        <x:v>User-owned original; permission confirmed</x:v>
+      </x:c>
       <x:c r="Q32" s="76" t="str">
-        <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Selected from IMG_0264.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
@@ -2599,13 +2615,13 @@
         <x:v>guardsman-pass.jpg</x:v>
       </x:c>
       <x:c r="H35" s="72" t="str">
-        <x:v>/images/passenger/around-you/wasatch-back.webp</x:v>
-      </x:c>
-      <x:c r="I35" s="78" t="str">
-        <x:v>Shared fallback</x:v>
-      </x:c>
-      <x:c r="J35" s="79" t="str">
-        <x:v>Yes</x:v>
+        <x:v>/images/passenger/around-you/user/guardsman-pass-juan.webp</x:v>
+      </x:c>
+      <x:c r="I35" s="74" t="str">
+        <x:v>Own local asset</x:v>
+      </x:c>
+      <x:c r="J35" s="75" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K35" s="72" t="n">
         <x:v>1</x:v>
@@ -2616,13 +2632,15 @@
       <x:c r="M35" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N35" s="72" t="str">
-        <x:v>https://www.fs.usda.gov/recarea/uwcnf/recarea/?recid=8982</x:v>
-      </x:c>
-      <x:c r="O35" s="72" t="str"/>
-      <x:c r="P35" s="72" t="str"/>
+      <x:c r="N35" s="72" t="str"/>
+      <x:c r="O35" s="72" t="str">
+        <x:v>STREEX-owned original — Juan</x:v>
+      </x:c>
+      <x:c r="P35" s="72" t="str">
+        <x:v>User-owned original; permission confirmed</x:v>
+      </x:c>
       <x:c r="Q35" s="72" t="str">
-        <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Selected from IMG_3408.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">

</xml_diff>

<commit_message>
Refresh Around You image assets
</commit_message>
<xml_diff>
--- a/assets-source/passenger/around-you/around-you-image-inventory.xlsx
+++ b/assets-source/passenger/around-you/around-you-image-inventory.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6e2087d121824cae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="Ra249ea74218041df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R5244dc85ab4e44c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="Rc49bc1cb6233491d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -772,8 +772,7 @@
         <x:v>Own local asset</x:v>
       </x:c>
       <x:c r="B14" s="33" t="n">
-        <x:f>COUNTIF('Inventory'!I5:I104,"Own local asset")</x:f>
-        <x:v>18</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C14" s="28"/>
       <x:c r="D14" s="28"/>
@@ -787,8 +786,7 @@
         <x:v>Original staged — rights recorded</x:v>
       </x:c>
       <x:c r="B15" s="33" t="n">
-        <x:f>COUNTIF('Inventory'!I5:I104,"Original staged — rights recorded")</x:f>
-        <x:v>6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C15" s="28"/>
       <x:c r="D15" s="28"/>
@@ -799,11 +797,10 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="37" t="str">
-        <x:v>Shared fallback</x:v>
+        <x:v>Curated Commons asset</x:v>
       </x:c>
       <x:c r="B16" s="33" t="n">
-        <x:f>COUNTIF('Inventory'!I5:I104,"Shared fallback")</x:f>
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="28"/>
@@ -814,11 +811,10 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="37" t="str">
-        <x:v>Missing original</x:v>
+        <x:v>Shared fallback</x:v>
       </x:c>
       <x:c r="B17" s="33" t="n">
-        <x:f>COUNTIF('Inventory'!I5:I104,"Missing original")</x:f>
-        <x:v>68</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C17" s="28"/>
       <x:c r="D17" s="28"/>
@@ -829,11 +825,10 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="37" t="str">
-        <x:v>Images still needed (active + candidates)</x:v>
+        <x:v>Missing original</x:v>
       </x:c>
       <x:c r="B18" s="33" t="n">
-        <x:f>COUNTIF('Inventory'!J5:J104,"Yes")</x:f>
-        <x:v>76</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C18" s="28"/>
       <x:c r="D18" s="28"/>
@@ -843,8 +838,12 @@
       <x:c r="H18" s="28"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="38"/>
-      <x:c r="B19" s="28"/>
+      <x:c r="A19" s="38" t="str">
+        <x:v>Images still needed</x:v>
+      </x:c>
+      <x:c r="B19" s="28" t="n">
+        <x:v>76</x:v>
+      </x:c>
       <x:c r="C19" s="28"/>
       <x:c r="D19" s="28"/>
       <x:c r="E19" s="28"/>
@@ -928,6 +927,14 @@
       </x:c>
       <x:c r="B25" s="25" t="str">
         <x:v>Planned place only; it is not enabled in the Passenger catalog yet.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>Curated Commons asset</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>Public WebP is bundled locally with source page, author and license recorded in the inventory.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1116,7 +1123,7 @@
       <x:c r="M5" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N5" s="72" t="str"/>
+      <x:c r="N5" s="72"/>
       <x:c r="O5" s="72" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1167,7 +1174,7 @@
       <x:c r="M6" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N6" s="76" t="str"/>
+      <x:c r="N6" s="76"/>
       <x:c r="O6" s="76" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1218,7 +1225,7 @@
       <x:c r="M7" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N7" s="72" t="str"/>
+      <x:c r="N7" s="72"/>
       <x:c r="O7" s="72" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1277,7 +1284,7 @@
         <x:v>User-owned original; permission confirmed</x:v>
       </x:c>
       <x:c r="Q8" s="76" t="str">
-        <x:v>Selected from IMG_0244.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
+        <x:v>Selected from renamed utah-state-capitol-night-gardens.jpeg; user-owned hero showing the Capitol grounds and dome, optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -1328,7 +1335,7 @@
         <x:v>User-owned original; permission confirmed</x:v>
       </x:c>
       <x:c r="Q9" s="72" t="str">
-        <x:v>Selected from IMG_0335.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
+        <x:v>Selected from renamed temple-square-night.jpeg; user-owned hero showing Temple Square architecture, optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
@@ -1371,7 +1378,7 @@
       <x:c r="M10" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N10" s="76" t="str"/>
+      <x:c r="N10" s="76"/>
       <x:c r="O10" s="76" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1422,7 +1429,7 @@
       <x:c r="M11" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N11" s="72" t="str"/>
+      <x:c r="N11" s="72"/>
       <x:c r="O11" s="72" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1455,9 +1462,11 @@
       <x:c r="G12" s="76" t="str">
         <x:v>university-of-utah.jpg</x:v>
       </x:c>
-      <x:c r="H12" s="76" t="str"/>
+      <x:c r="H12" s="76" t="str">
+        <x:v>/images/passenger/around-you/curated/university-of-utah-campus.webp</x:v>
+      </x:c>
       <x:c r="I12" s="77" t="str">
-        <x:v>Original staged — rights recorded</x:v>
+        <x:v>Curated Commons asset</x:v>
       </x:c>
       <x:c r="J12" s="75" t="str">
         <x:v>No</x:v>
@@ -1472,16 +1481,16 @@
         <x:v>Active coordinates</x:v>
       </x:c>
       <x:c r="N12" s="76" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:University_of_Utah_campus.jpg</x:v>
+        <x:v>https://commons.wikimedia.org/wiki/File:University_of_Utah_Presidents_Circle_.jpg</x:v>
       </x:c>
       <x:c r="O12" s="76" t="str">
-        <x:v>Wikimedia Commons — SounderBruce from Seattle, United States</x:v>
+        <x:v>Wikimedia Commons — MrSchmidt</x:v>
       </x:c>
       <x:c r="P12" s="76" t="str">
-        <x:v>CC BY-SA 2.0 — attribution and share-alike required</x:v>
+        <x:v>CC BY-SA 4.0 — attribution and share-alike required</x:v>
       </x:c>
       <x:c r="Q12" s="76" t="str">
-        <x:v>Original staged in assets-source/passenger/around-you; rights recorded. Optimize/crop to public WebP in P1.3. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Curated from utah-presidents-circle.jpg; cropped and optimized to metadata-free WebP with the campus architecture clearly visible.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -1506,9 +1515,11 @@
       <x:c r="G13" s="72" t="str">
         <x:v>red-butte-garden.jpg</x:v>
       </x:c>
-      <x:c r="H13" s="72" t="str"/>
+      <x:c r="H13" s="72" t="str">
+        <x:v>/images/passenger/around-you/curated/red-butte-garden.webp</x:v>
+      </x:c>
       <x:c r="I13" s="77" t="str">
-        <x:v>Original staged — rights recorded</x:v>
+        <x:v>Curated Commons asset</x:v>
       </x:c>
       <x:c r="J13" s="75" t="str">
         <x:v>No</x:v>
@@ -1523,16 +1534,16 @@
         <x:v>Active coordinates</x:v>
       </x:c>
       <x:c r="N13" s="72" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:Entry_-_Red_Butte_Garden_and_Arboretum_-_DSC07474.JPG</x:v>
+        <x:v>https://commons.wikimedia.org/wiki/File:Red_Butte_Garden2.jpg</x:v>
       </x:c>
       <x:c r="O13" s="72" t="str">
-        <x:v>Wikimedia Commons — Daderot</x:v>
+        <x:v>Wikimedia Commons — C.Maylett</x:v>
       </x:c>
       <x:c r="P13" s="72" t="str">
-        <x:v>CC0 — no attribution required; attribution retained in inventory</x:v>
+        <x:v>CC BY-SA 3.0 — attribution and share-alike required</x:v>
       </x:c>
       <x:c r="Q13" s="72" t="str">
-        <x:v>Original staged in assets-source/passenger/around-you; rights recorded. Optimize/crop to public WebP in P1.3. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Curated garden interior image; optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
@@ -1557,7 +1568,7 @@
       <x:c r="G14" s="76" t="str">
         <x:v>this-is-the-place.jpg</x:v>
       </x:c>
-      <x:c r="H14" s="76" t="str"/>
+      <x:c r="H14" s="76"/>
       <x:c r="I14" s="77" t="str">
         <x:v>Original staged — rights recorded</x:v>
       </x:c>
@@ -1608,9 +1619,11 @@
       <x:c r="G15" s="72" t="str">
         <x:v>salt-lake-city-airport.jpg</x:v>
       </x:c>
-      <x:c r="H15" s="72" t="str"/>
+      <x:c r="H15" s="72" t="str">
+        <x:v>/images/passenger/around-you/curated/salt-lake-city-airport-terminal.webp</x:v>
+      </x:c>
       <x:c r="I15" s="77" t="str">
-        <x:v>Original staged — rights recorded</x:v>
+        <x:v>Curated Commons asset</x:v>
       </x:c>
       <x:c r="J15" s="75" t="str">
         <x:v>No</x:v>
@@ -1625,16 +1638,16 @@
         <x:v>Active coordinates</x:v>
       </x:c>
       <x:c r="N15" s="72" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:Salt_Lake_City_International_Airport_SLC.jpg</x:v>
+        <x:v>https://commons.wikimedia.org/wiki/File:2015-04-14_00_11_43_View_towards_the_International_Terminal_and_Concourse_D_from_the_inner_end_of_Concourse_C_in_Salt_Lake_City_International_Airport,_Utah.jpg</x:v>
       </x:c>
       <x:c r="O15" s="72" t="str">
-        <x:v>Wikimedia Commons — Ron Reiring</x:v>
+        <x:v>Wikimedia Commons — Famartin</x:v>
       </x:c>
       <x:c r="P15" s="72" t="str">
-        <x:v>CC BY 2.0 — attribution required</x:v>
+        <x:v>CC BY-SA 4.0 — attribution and share-alike required</x:v>
       </x:c>
       <x:c r="Q15" s="72" t="str">
-        <x:v>Original staged in assets-source/passenger/around-you; rights recorded. Optimize/crop to public WebP in P1.3. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
+        <x:v>Curated terminal/interior view rather than an aerial; optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
@@ -1677,7 +1690,7 @@
       <x:c r="M16" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N16" s="76" t="str"/>
+      <x:c r="N16" s="76"/>
       <x:c r="O16" s="76" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1710,7 +1723,7 @@
       <x:c r="G17" s="72" t="str">
         <x:v>parleys-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H17" s="72" t="str"/>
+      <x:c r="H17" s="72"/>
       <x:c r="I17" s="77" t="str">
         <x:v>Original staged — rights recorded</x:v>
       </x:c>
@@ -1762,10 +1775,10 @@
         <x:v>lagoon-amusement-park.jpg</x:v>
       </x:c>
       <x:c r="H18" s="76" t="str">
-        <x:v>/images/passenger/around-you/user/lagoon-amusement-park-juan.webp</x:v>
+        <x:v>/images/passenger/around-you/curated/lagoon-exterior.webp</x:v>
       </x:c>
       <x:c r="I18" s="74" t="str">
-        <x:v>Own local asset</x:v>
+        <x:v>Curated Commons asset</x:v>
       </x:c>
       <x:c r="J18" s="75" t="str">
         <x:v>No</x:v>
@@ -1779,15 +1792,17 @@
       <x:c r="M18" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N18" s="76" t="str"/>
+      <x:c r="N18" s="76" t="str">
+        <x:v>https://commons.wikimedia.org/wiki/File:Lagoon_Roller_Coaster_winter.jpeg</x:v>
+      </x:c>
       <x:c r="O18" s="76" t="str">
-        <x:v>STREEX-owned original — Juan</x:v>
+        <x:v>Wikimedia Commons — Ntsimp</x:v>
       </x:c>
       <x:c r="P18" s="76" t="str">
-        <x:v>User-owned original; permission confirmed</x:v>
+        <x:v>CC0 — no attribution required</x:v>
       </x:c>
       <x:c r="Q18" s="76" t="str">
-        <x:v>Selected from IMG_2568.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
+        <x:v>Curated exterior attraction view; optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
@@ -1812,7 +1827,7 @@
       <x:c r="G19" s="72" t="str">
         <x:v>ogden.jpg</x:v>
       </x:c>
-      <x:c r="H19" s="72" t="str"/>
+      <x:c r="H19" s="72"/>
       <x:c r="I19" s="77" t="str">
         <x:v>Original staged — rights recorded</x:v>
       </x:c>
@@ -1881,7 +1896,7 @@
       <x:c r="M20" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N20" s="76" t="str"/>
+      <x:c r="N20" s="76"/>
       <x:c r="O20" s="76" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1932,7 +1947,7 @@
       <x:c r="M21" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N21" s="72" t="str"/>
+      <x:c r="N21" s="72"/>
       <x:c r="O21" s="72" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1983,7 +1998,7 @@
       <x:c r="M22" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N22" s="76" t="str"/>
+      <x:c r="N22" s="76"/>
       <x:c r="O22" s="76" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -2034,7 +2049,7 @@
       <x:c r="M23" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N23" s="72" t="str"/>
+      <x:c r="N23" s="72"/>
       <x:c r="O23" s="72" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -2068,10 +2083,10 @@
         <x:v>kimball-junction.jpg</x:v>
       </x:c>
       <x:c r="H24" s="76" t="str">
-        <x:v>/images/passenger/around-you/user/kimball-junction-juan.webp</x:v>
+        <x:v>/images/passenger/around-you/curated/kimball-junction-sunset.webp</x:v>
       </x:c>
       <x:c r="I24" s="74" t="str">
-        <x:v>Own local asset</x:v>
+        <x:v>Curated Commons asset</x:v>
       </x:c>
       <x:c r="J24" s="75" t="str">
         <x:v>No</x:v>
@@ -2085,15 +2100,17 @@
       <x:c r="M24" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N24" s="76" t="str"/>
+      <x:c r="N24" s="76" t="str">
+        <x:v>https://commons.wikimedia.org/wiki/File:Kimball_Junction,_United_States_(Unsplash).jpg</x:v>
+      </x:c>
       <x:c r="O24" s="76" t="str">
-        <x:v>STREEX-owned original — Juan</x:v>
+        <x:v>Wikimedia Commons — Patrick Hendry</x:v>
       </x:c>
       <x:c r="P24" s="76" t="str">
-        <x:v>User-owned original; permission confirmed</x:v>
+        <x:v>CC0 — no attribution required</x:v>
       </x:c>
       <x:c r="Q24" s="76" t="str">
-        <x:v>Selected from IMG_4721.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
+        <x:v>Curated sunset view for the Kimball Junction corridor; optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
@@ -2136,7 +2153,7 @@
       <x:c r="M25" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N25" s="72" t="str"/>
+      <x:c r="N25" s="72"/>
       <x:c r="O25" s="72" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -2190,8 +2207,8 @@
       <x:c r="N26" s="76" t="str">
         <x:v>https://nhmu.utah.edu/</x:v>
       </x:c>
-      <x:c r="O26" s="76" t="str"/>
-      <x:c r="P26" s="76" t="str"/>
+      <x:c r="O26" s="76"/>
+      <x:c r="P26" s="76"/>
       <x:c r="Q26" s="76" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2239,8 +2256,8 @@
       <x:c r="N27" s="72" t="str">
         <x:v>https://www.slc.gov/parks/parks-division/ensign-peak-nature-park/</x:v>
       </x:c>
-      <x:c r="O27" s="72" t="str"/>
-      <x:c r="P27" s="72" t="str"/>
+      <x:c r="O27" s="72"/>
+      <x:c r="P27" s="72"/>
       <x:c r="Q27" s="72" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2288,8 +2305,8 @@
       <x:c r="N28" s="76" t="str">
         <x:v>https://tracyaviary.org/</x:v>
       </x:c>
-      <x:c r="O28" s="76" t="str"/>
-      <x:c r="P28" s="76" t="str"/>
+      <x:c r="O28" s="76"/>
+      <x:c r="P28" s="76"/>
       <x:c r="Q28" s="76" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2337,8 +2354,8 @@
       <x:c r="N29" s="72" t="str">
         <x:v>https://www.hoglezoo.org/</x:v>
       </x:c>
-      <x:c r="O29" s="72" t="str"/>
-      <x:c r="P29" s="72" t="str"/>
+      <x:c r="O29" s="72"/>
+      <x:c r="P29" s="72"/>
       <x:c r="Q29" s="72" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2383,7 +2400,7 @@
       <x:c r="M30" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N30" s="76" t="str"/>
+      <x:c r="N30" s="76"/>
       <x:c r="O30" s="76" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -2437,8 +2454,8 @@
       <x:c r="N31" s="72" t="str">
         <x:v>https://www.slc.gov/parks/parks-division/gilgal-sculpture-garden/</x:v>
       </x:c>
-      <x:c r="O31" s="72" t="str"/>
-      <x:c r="P31" s="72" t="str"/>
+      <x:c r="O31" s="72"/>
+      <x:c r="P31" s="72"/>
       <x:c r="Q31" s="72" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2483,7 +2500,7 @@
       <x:c r="M32" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N32" s="76" t="str"/>
+      <x:c r="N32" s="76"/>
       <x:c r="O32" s="76" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -2537,8 +2554,8 @@
       <x:c r="N33" s="72" t="str">
         <x:v>https://www.parkcity.org/departments/trails-open-space/historic-mcpolin-barn</x:v>
       </x:c>
-      <x:c r="O33" s="72" t="str"/>
-      <x:c r="P33" s="72" t="str"/>
+      <x:c r="O33" s="72"/>
+      <x:c r="P33" s="72"/>
       <x:c r="Q33" s="72" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2586,8 +2603,8 @@
       <x:c r="N34" s="76" t="str">
         <x:v>https://stateparks.utah.gov/parks/jordanelle/</x:v>
       </x:c>
-      <x:c r="O34" s="76" t="str"/>
-      <x:c r="P34" s="76" t="str"/>
+      <x:c r="O34" s="76"/>
+      <x:c r="P34" s="76"/>
       <x:c r="Q34" s="76" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2632,7 +2649,7 @@
       <x:c r="M35" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N35" s="72" t="str"/>
+      <x:c r="N35" s="72"/>
       <x:c r="O35" s="72" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -2686,8 +2703,8 @@
       <x:c r="N36" s="76" t="str">
         <x:v>https://www.egyptiantheatrecompany.org/</x:v>
       </x:c>
-      <x:c r="O36" s="76" t="str"/>
-      <x:c r="P36" s="76" t="str"/>
+      <x:c r="O36" s="76"/>
+      <x:c r="P36" s="76"/>
       <x:c r="Q36" s="76" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2714,7 +2731,7 @@
       <x:c r="G37" s="72" t="str">
         <x:v>utah-museum-of-fine-arts.jpg</x:v>
       </x:c>
-      <x:c r="H37" s="72" t="str"/>
+      <x:c r="H37" s="72"/>
       <x:c r="I37" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -2733,8 +2750,8 @@
       <x:c r="N37" s="72" t="str">
         <x:v>https://www.umfa.utah.edu/</x:v>
       </x:c>
-      <x:c r="O37" s="72" t="str"/>
-      <x:c r="P37" s="72" t="str"/>
+      <x:c r="O37" s="72"/>
+      <x:c r="P37" s="72"/>
       <x:c r="Q37" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2761,7 +2778,7 @@
       <x:c r="G38" s="76" t="str">
         <x:v>the-leonardo.jpg</x:v>
       </x:c>
-      <x:c r="H38" s="76" t="str"/>
+      <x:c r="H38" s="76"/>
       <x:c r="I38" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -2780,8 +2797,8 @@
       <x:c r="N38" s="76" t="str">
         <x:v>https://theleonardo.org/</x:v>
       </x:c>
-      <x:c r="O38" s="76" t="str"/>
-      <x:c r="P38" s="76" t="str"/>
+      <x:c r="O38" s="76"/>
+      <x:c r="P38" s="76"/>
       <x:c r="Q38" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2808,7 +2825,7 @@
       <x:c r="G39" s="72" t="str">
         <x:v>clark-planetarium.jpg</x:v>
       </x:c>
-      <x:c r="H39" s="72" t="str"/>
+      <x:c r="H39" s="72"/>
       <x:c r="I39" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -2827,8 +2844,8 @@
       <x:c r="N39" s="72" t="str">
         <x:v>https://slplanet.com/</x:v>
       </x:c>
-      <x:c r="O39" s="72" t="str"/>
-      <x:c r="P39" s="72" t="str"/>
+      <x:c r="O39" s="72"/>
+      <x:c r="P39" s="72"/>
       <x:c r="Q39" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2855,7 +2872,7 @@
       <x:c r="G40" s="76" t="str">
         <x:v>discovery-gateway.jpg</x:v>
       </x:c>
-      <x:c r="H40" s="76" t="str"/>
+      <x:c r="H40" s="76"/>
       <x:c r="I40" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -2874,8 +2891,8 @@
       <x:c r="N40" s="76" t="str">
         <x:v>https://discoverygateway.org/</x:v>
       </x:c>
-      <x:c r="O40" s="76" t="str"/>
-      <x:c r="P40" s="76" t="str"/>
+      <x:c r="O40" s="76"/>
+      <x:c r="P40" s="76"/>
       <x:c r="Q40" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2902,7 +2919,7 @@
       <x:c r="G41" s="72" t="str">
         <x:v>salt-palace-convention-center.jpg</x:v>
       </x:c>
-      <x:c r="H41" s="72" t="str"/>
+      <x:c r="H41" s="72"/>
       <x:c r="I41" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -2921,8 +2938,8 @@
       <x:c r="N41" s="72" t="str">
         <x:v>https://www.visitsaltlake.com/</x:v>
       </x:c>
-      <x:c r="O41" s="72" t="str"/>
-      <x:c r="P41" s="72" t="str"/>
+      <x:c r="O41" s="72"/>
+      <x:c r="P41" s="72"/>
       <x:c r="Q41" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2949,7 +2966,7 @@
       <x:c r="G42" s="76" t="str">
         <x:v>eccles-theater.jpg</x:v>
       </x:c>
-      <x:c r="H42" s="76" t="str"/>
+      <x:c r="H42" s="76"/>
       <x:c r="I42" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -2968,8 +2985,8 @@
       <x:c r="N42" s="76" t="str">
         <x:v>https://www.eccles-theater.com/</x:v>
       </x:c>
-      <x:c r="O42" s="76" t="str"/>
-      <x:c r="P42" s="76" t="str"/>
+      <x:c r="O42" s="76"/>
+      <x:c r="P42" s="76"/>
       <x:c r="Q42" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2996,7 +3013,7 @@
       <x:c r="G43" s="72" t="str">
         <x:v>abravanel-hall.jpg</x:v>
       </x:c>
-      <x:c r="H43" s="72" t="str"/>
+      <x:c r="H43" s="72"/>
       <x:c r="I43" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3015,8 +3032,8 @@
       <x:c r="N43" s="72" t="str">
         <x:v>https://utaharts.org/</x:v>
       </x:c>
-      <x:c r="O43" s="72" t="str"/>
-      <x:c r="P43" s="72" t="str"/>
+      <x:c r="O43" s="72"/>
+      <x:c r="P43" s="72"/>
       <x:c r="Q43" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3043,7 +3060,7 @@
       <x:c r="G44" s="76" t="str">
         <x:v>delta-center.jpg</x:v>
       </x:c>
-      <x:c r="H44" s="76" t="str"/>
+      <x:c r="H44" s="76"/>
       <x:c r="I44" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3062,8 +3079,8 @@
       <x:c r="N44" s="76" t="str">
         <x:v>https://www.nba.com/jazz/arena</x:v>
       </x:c>
-      <x:c r="O44" s="76" t="str"/>
-      <x:c r="P44" s="76" t="str"/>
+      <x:c r="O44" s="76"/>
+      <x:c r="P44" s="76"/>
       <x:c r="Q44" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3090,7 +3107,7 @@
       <x:c r="G45" s="72" t="str">
         <x:v>rice-eccles-stadium.jpg</x:v>
       </x:c>
-      <x:c r="H45" s="72" t="str"/>
+      <x:c r="H45" s="72"/>
       <x:c r="I45" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3109,8 +3126,8 @@
       <x:c r="N45" s="72" t="str">
         <x:v>https://stadium.utah.edu/</x:v>
       </x:c>
-      <x:c r="O45" s="72" t="str"/>
-      <x:c r="P45" s="72" t="str"/>
+      <x:c r="O45" s="72"/>
+      <x:c r="P45" s="72"/>
       <x:c r="Q45" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3137,7 +3154,7 @@
       <x:c r="G46" s="76" t="str">
         <x:v>america-first-field.jpg</x:v>
       </x:c>
-      <x:c r="H46" s="76" t="str"/>
+      <x:c r="H46" s="76"/>
       <x:c r="I46" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3156,8 +3173,8 @@
       <x:c r="N46" s="76" t="str">
         <x:v>https://www.rsl.com/america-first-field</x:v>
       </x:c>
-      <x:c r="O46" s="76" t="str"/>
-      <x:c r="P46" s="76" t="str"/>
+      <x:c r="O46" s="76"/>
+      <x:c r="P46" s="76"/>
       <x:c r="Q46" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3184,7 +3201,7 @@
       <x:c r="G47" s="72" t="str">
         <x:v>maverik-stadium.jpg</x:v>
       </x:c>
-      <x:c r="H47" s="72" t="str"/>
+      <x:c r="H47" s="72"/>
       <x:c r="I47" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3203,8 +3220,8 @@
       <x:c r="N47" s="72" t="str">
         <x:v>https://utahstateaggies.com/facilities/maverik-stadium/</x:v>
       </x:c>
-      <x:c r="O47" s="72" t="str"/>
-      <x:c r="P47" s="72" t="str"/>
+      <x:c r="O47" s="72"/>
+      <x:c r="P47" s="72"/>
       <x:c r="Q47" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3231,7 +3248,7 @@
       <x:c r="G48" s="76" t="str">
         <x:v>utah-state-fairpark.jpg</x:v>
       </x:c>
-      <x:c r="H48" s="76" t="str"/>
+      <x:c r="H48" s="76"/>
       <x:c r="I48" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3250,8 +3267,8 @@
       <x:c r="N48" s="76" t="str">
         <x:v>https://utahstatefair.com/</x:v>
       </x:c>
-      <x:c r="O48" s="76" t="str"/>
-      <x:c r="P48" s="76" t="str"/>
+      <x:c r="O48" s="76"/>
+      <x:c r="P48" s="76"/>
       <x:c r="Q48" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3278,7 +3295,7 @@
       <x:c r="G49" s="72" t="str">
         <x:v>sugar-house-park.jpg</x:v>
       </x:c>
-      <x:c r="H49" s="72" t="str"/>
+      <x:c r="H49" s="72"/>
       <x:c r="I49" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3297,8 +3314,8 @@
       <x:c r="N49" s="72" t="str">
         <x:v>https://www.slc.gov/parks/</x:v>
       </x:c>
-      <x:c r="O49" s="72" t="str"/>
-      <x:c r="P49" s="72" t="str"/>
+      <x:c r="O49" s="72"/>
+      <x:c r="P49" s="72"/>
       <x:c r="Q49" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3325,7 +3342,7 @@
       <x:c r="G50" s="76" t="str">
         <x:v>9th-and-9th.jpg</x:v>
       </x:c>
-      <x:c r="H50" s="76" t="str"/>
+      <x:c r="H50" s="76"/>
       <x:c r="I50" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3344,8 +3361,8 @@
       <x:c r="N50" s="76" t="str">
         <x:v>https://www.visitsaltlake.com/</x:v>
       </x:c>
-      <x:c r="O50" s="76" t="str"/>
-      <x:c r="P50" s="76" t="str"/>
+      <x:c r="O50" s="76"/>
+      <x:c r="P50" s="76"/>
       <x:c r="Q50" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3372,7 +3389,7 @@
       <x:c r="G51" s="72" t="str">
         <x:v>the-avenues.jpg</x:v>
       </x:c>
-      <x:c r="H51" s="72" t="str"/>
+      <x:c r="H51" s="72"/>
       <x:c r="I51" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3391,8 +3408,8 @@
       <x:c r="N51" s="72" t="str">
         <x:v>https://www.slc.gov/</x:v>
       </x:c>
-      <x:c r="O51" s="72" t="str"/>
-      <x:c r="P51" s="72" t="str"/>
+      <x:c r="O51" s="72"/>
+      <x:c r="P51" s="72"/>
       <x:c r="Q51" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3419,7 +3436,7 @@
       <x:c r="G52" s="76" t="str">
         <x:v>memory-grove-park.jpg</x:v>
       </x:c>
-      <x:c r="H52" s="76" t="str"/>
+      <x:c r="H52" s="76"/>
       <x:c r="I52" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3438,8 +3455,8 @@
       <x:c r="N52" s="76" t="str">
         <x:v>https://www.slc.gov/parks/</x:v>
       </x:c>
-      <x:c r="O52" s="76" t="str"/>
-      <x:c r="P52" s="76" t="str"/>
+      <x:c r="O52" s="76"/>
+      <x:c r="P52" s="76"/>
       <x:c r="Q52" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3466,7 +3483,7 @@
       <x:c r="G53" s="72" t="str">
         <x:v>jordan-river-parkway.jpg</x:v>
       </x:c>
-      <x:c r="H53" s="72" t="str"/>
+      <x:c r="H53" s="72"/>
       <x:c r="I53" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3485,8 +3502,8 @@
       <x:c r="N53" s="72" t="str">
         <x:v>https://www.slc.gov/parks/</x:v>
       </x:c>
-      <x:c r="O53" s="72" t="str"/>
-      <x:c r="P53" s="72" t="str"/>
+      <x:c r="O53" s="72"/>
+      <x:c r="P53" s="72"/>
       <x:c r="Q53" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3513,7 +3530,7 @@
       <x:c r="G54" s="76" t="str">
         <x:v>bonneville-shoreline-trail.jpg</x:v>
       </x:c>
-      <x:c r="H54" s="76" t="str"/>
+      <x:c r="H54" s="76"/>
       <x:c r="I54" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3532,8 +3549,8 @@
       <x:c r="N54" s="76" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O54" s="76" t="str"/>
-      <x:c r="P54" s="76" t="str"/>
+      <x:c r="O54" s="76"/>
+      <x:c r="P54" s="76"/>
       <x:c r="Q54" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3560,7 +3577,7 @@
       <x:c r="G55" s="72" t="str">
         <x:v>big-cottonwood-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H55" s="72" t="str"/>
+      <x:c r="H55" s="72"/>
       <x:c r="I55" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3579,8 +3596,8 @@
       <x:c r="N55" s="72" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O55" s="72" t="str"/>
-      <x:c r="P55" s="72" t="str"/>
+      <x:c r="O55" s="72"/>
+      <x:c r="P55" s="72"/>
       <x:c r="Q55" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3607,7 +3624,7 @@
       <x:c r="G56" s="76" t="str">
         <x:v>little-cottonwood-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H56" s="76" t="str"/>
+      <x:c r="H56" s="76"/>
       <x:c r="I56" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3626,8 +3643,8 @@
       <x:c r="N56" s="76" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O56" s="76" t="str"/>
-      <x:c r="P56" s="76" t="str"/>
+      <x:c r="O56" s="76"/>
+      <x:c r="P56" s="76"/>
       <x:c r="Q56" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3654,7 +3671,7 @@
       <x:c r="G57" s="72" t="str">
         <x:v>millcreek-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H57" s="72" t="str"/>
+      <x:c r="H57" s="72"/>
       <x:c r="I57" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3673,8 +3690,8 @@
       <x:c r="N57" s="72" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O57" s="72" t="str"/>
-      <x:c r="P57" s="72" t="str"/>
+      <x:c r="O57" s="72"/>
+      <x:c r="P57" s="72"/>
       <x:c r="Q57" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3701,7 +3718,7 @@
       <x:c r="G58" s="76" t="str">
         <x:v>snowbird.jpg</x:v>
       </x:c>
-      <x:c r="H58" s="76" t="str"/>
+      <x:c r="H58" s="76"/>
       <x:c r="I58" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3720,8 +3737,8 @@
       <x:c r="N58" s="76" t="str">
         <x:v>https://www.snowbird.com/</x:v>
       </x:c>
-      <x:c r="O58" s="76" t="str"/>
-      <x:c r="P58" s="76" t="str"/>
+      <x:c r="O58" s="76"/>
+      <x:c r="P58" s="76"/>
       <x:c r="Q58" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3748,7 +3765,7 @@
       <x:c r="G59" s="72" t="str">
         <x:v>alta-ski-area.jpg</x:v>
       </x:c>
-      <x:c r="H59" s="72" t="str"/>
+      <x:c r="H59" s="72"/>
       <x:c r="I59" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3767,8 +3784,8 @@
       <x:c r="N59" s="72" t="str">
         <x:v>https://www.alta.com/</x:v>
       </x:c>
-      <x:c r="O59" s="72" t="str"/>
-      <x:c r="P59" s="72" t="str"/>
+      <x:c r="O59" s="72"/>
+      <x:c r="P59" s="72"/>
       <x:c r="Q59" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3795,7 +3812,7 @@
       <x:c r="G60" s="76" t="str">
         <x:v>solitude-mountain-resort.jpg</x:v>
       </x:c>
-      <x:c r="H60" s="76" t="str"/>
+      <x:c r="H60" s="76"/>
       <x:c r="I60" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3814,8 +3831,8 @@
       <x:c r="N60" s="76" t="str">
         <x:v>https://www.solitudemountain.com/</x:v>
       </x:c>
-      <x:c r="O60" s="76" t="str"/>
-      <x:c r="P60" s="76" t="str"/>
+      <x:c r="O60" s="76"/>
+      <x:c r="P60" s="76"/>
       <x:c r="Q60" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3842,7 +3859,7 @@
       <x:c r="G61" s="72" t="str">
         <x:v>brighton-resort.jpg</x:v>
       </x:c>
-      <x:c r="H61" s="72" t="str"/>
+      <x:c r="H61" s="72"/>
       <x:c r="I61" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3861,8 +3878,8 @@
       <x:c r="N61" s="72" t="str">
         <x:v>https://brightonresort.com/</x:v>
       </x:c>
-      <x:c r="O61" s="72" t="str"/>
-      <x:c r="P61" s="72" t="str"/>
+      <x:c r="O61" s="72"/>
+      <x:c r="P61" s="72"/>
       <x:c r="Q61" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3889,7 +3906,7 @@
       <x:c r="G62" s="76" t="str">
         <x:v>snowbasin-resort.jpg</x:v>
       </x:c>
-      <x:c r="H62" s="76" t="str"/>
+      <x:c r="H62" s="76"/>
       <x:c r="I62" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3908,8 +3925,8 @@
       <x:c r="N62" s="76" t="str">
         <x:v>https://www.snowbasin.com/</x:v>
       </x:c>
-      <x:c r="O62" s="76" t="str"/>
-      <x:c r="P62" s="76" t="str"/>
+      <x:c r="O62" s="76"/>
+      <x:c r="P62" s="76"/>
       <x:c r="Q62" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3936,7 +3953,7 @@
       <x:c r="G63" s="72" t="str">
         <x:v>powder-mountain.jpg</x:v>
       </x:c>
-      <x:c r="H63" s="72" t="str"/>
+      <x:c r="H63" s="72"/>
       <x:c r="I63" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -3955,8 +3972,8 @@
       <x:c r="N63" s="72" t="str">
         <x:v>https://www.powdermountain.com/</x:v>
       </x:c>
-      <x:c r="O63" s="72" t="str"/>
-      <x:c r="P63" s="72" t="str"/>
+      <x:c r="O63" s="72"/>
+      <x:c r="P63" s="72"/>
       <x:c r="Q63" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3983,7 +4000,7 @@
       <x:c r="G64" s="76" t="str">
         <x:v>canyons-village.jpg</x:v>
       </x:c>
-      <x:c r="H64" s="76" t="str"/>
+      <x:c r="H64" s="76"/>
       <x:c r="I64" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4002,8 +4019,8 @@
       <x:c r="N64" s="76" t="str">
         <x:v>https://www.visitparkcity.com/</x:v>
       </x:c>
-      <x:c r="O64" s="76" t="str"/>
-      <x:c r="P64" s="76" t="str"/>
+      <x:c r="O64" s="76"/>
+      <x:c r="P64" s="76"/>
       <x:c r="Q64" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4030,7 +4047,7 @@
       <x:c r="G65" s="72" t="str">
         <x:v>park-city-mountain.jpg</x:v>
       </x:c>
-      <x:c r="H65" s="72" t="str"/>
+      <x:c r="H65" s="72"/>
       <x:c r="I65" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4049,8 +4066,8 @@
       <x:c r="N65" s="72" t="str">
         <x:v>https://www.visitparkcity.com/</x:v>
       </x:c>
-      <x:c r="O65" s="72" t="str"/>
-      <x:c r="P65" s="72" t="str"/>
+      <x:c r="O65" s="72"/>
+      <x:c r="P65" s="72"/>
       <x:c r="Q65" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4077,7 +4094,7 @@
       <x:c r="G66" s="76" t="str">
         <x:v>park-city-library.jpg</x:v>
       </x:c>
-      <x:c r="H66" s="76" t="str"/>
+      <x:c r="H66" s="76"/>
       <x:c r="I66" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4096,8 +4113,8 @@
       <x:c r="N66" s="76" t="str">
         <x:v>https://www.visitparkcity.com/</x:v>
       </x:c>
-      <x:c r="O66" s="76" t="str"/>
-      <x:c r="P66" s="76" t="str"/>
+      <x:c r="O66" s="76"/>
+      <x:c r="P66" s="76"/>
       <x:c r="Q66" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4124,7 +4141,7 @@
       <x:c r="G67" s="72" t="str">
         <x:v>park-city-museum.jpg</x:v>
       </x:c>
-      <x:c r="H67" s="72" t="str"/>
+      <x:c r="H67" s="72"/>
       <x:c r="I67" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4143,8 +4160,8 @@
       <x:c r="N67" s="72" t="str">
         <x:v>https://www.parkcityhistory.org/</x:v>
       </x:c>
-      <x:c r="O67" s="72" t="str"/>
-      <x:c r="P67" s="72" t="str"/>
+      <x:c r="O67" s="72"/>
+      <x:c r="P67" s="72"/>
       <x:c r="Q67" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4171,7 +4188,7 @@
       <x:c r="G68" s="76" t="str">
         <x:v>woodward-park-city.jpg</x:v>
       </x:c>
-      <x:c r="H68" s="76" t="str"/>
+      <x:c r="H68" s="76"/>
       <x:c r="I68" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4190,8 +4207,8 @@
       <x:c r="N68" s="76" t="str">
         <x:v>https://woodwardparkcity.com/</x:v>
       </x:c>
-      <x:c r="O68" s="76" t="str"/>
-      <x:c r="P68" s="76" t="str"/>
+      <x:c r="O68" s="76"/>
+      <x:c r="P68" s="76"/>
       <x:c r="Q68" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4218,7 +4235,7 @@
       <x:c r="G69" s="72" t="str">
         <x:v>heber-valley-railroad.jpg</x:v>
       </x:c>
-      <x:c r="H69" s="72" t="str"/>
+      <x:c r="H69" s="72"/>
       <x:c r="I69" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4237,8 +4254,8 @@
       <x:c r="N69" s="72" t="str">
         <x:v>https://www.hebervalleyrr.org/</x:v>
       </x:c>
-      <x:c r="O69" s="72" t="str"/>
-      <x:c r="P69" s="72" t="str"/>
+      <x:c r="O69" s="72"/>
+      <x:c r="P69" s="72"/>
       <x:c r="Q69" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4265,7 +4282,7 @@
       <x:c r="G70" s="76" t="str">
         <x:v>deer-creek-reservoir.jpg</x:v>
       </x:c>
-      <x:c r="H70" s="76" t="str"/>
+      <x:c r="H70" s="76"/>
       <x:c r="I70" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4284,8 +4301,8 @@
       <x:c r="N70" s="76" t="str">
         <x:v>https://stateparks.utah.gov/</x:v>
       </x:c>
-      <x:c r="O70" s="76" t="str"/>
-      <x:c r="P70" s="76" t="str"/>
+      <x:c r="O70" s="76"/>
+      <x:c r="P70" s="76"/>
       <x:c r="Q70" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4312,7 +4329,7 @@
       <x:c r="G71" s="72" t="str">
         <x:v>provo-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H71" s="72" t="str"/>
+      <x:c r="H71" s="72"/>
       <x:c r="I71" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4331,8 +4348,8 @@
       <x:c r="N71" s="72" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O71" s="72" t="str"/>
-      <x:c r="P71" s="72" t="str"/>
+      <x:c r="O71" s="72"/>
+      <x:c r="P71" s="72"/>
       <x:c r="Q71" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4359,7 +4376,7 @@
       <x:c r="G72" s="76" t="str">
         <x:v>bridal-veil-falls.jpg</x:v>
       </x:c>
-      <x:c r="H72" s="76" t="str"/>
+      <x:c r="H72" s="76"/>
       <x:c r="I72" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4378,8 +4395,8 @@
       <x:c r="N72" s="76" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O72" s="76" t="str"/>
-      <x:c r="P72" s="76" t="str"/>
+      <x:c r="O72" s="76"/>
+      <x:c r="P72" s="76"/>
       <x:c r="Q72" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4406,7 +4423,7 @@
       <x:c r="G73" s="72" t="str">
         <x:v>mount-timpanogos.jpg</x:v>
       </x:c>
-      <x:c r="H73" s="72" t="str"/>
+      <x:c r="H73" s="72"/>
       <x:c r="I73" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4425,8 +4442,8 @@
       <x:c r="N73" s="72" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O73" s="72" t="str"/>
-      <x:c r="P73" s="72" t="str"/>
+      <x:c r="O73" s="72"/>
+      <x:c r="P73" s="72"/>
       <x:c r="Q73" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4453,7 +4470,7 @@
       <x:c r="G74" s="76" t="str">
         <x:v>ogden-union-station.jpg</x:v>
       </x:c>
-      <x:c r="H74" s="76" t="str"/>
+      <x:c r="H74" s="76"/>
       <x:c r="I74" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4472,8 +4489,8 @@
       <x:c r="N74" s="76" t="str">
         <x:v>https://www.visitogden.com/</x:v>
       </x:c>
-      <x:c r="O74" s="76" t="str"/>
-      <x:c r="P74" s="76" t="str"/>
+      <x:c r="O74" s="76"/>
+      <x:c r="P74" s="76"/>
       <x:c r="Q74" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4500,7 +4517,7 @@
       <x:c r="G75" s="72" t="str">
         <x:v>eccles-dinosaur-park.jpg</x:v>
       </x:c>
-      <x:c r="H75" s="72" t="str"/>
+      <x:c r="H75" s="72"/>
       <x:c r="I75" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4519,8 +4536,8 @@
       <x:c r="N75" s="72" t="str">
         <x:v>https://dinosaurpark.org/</x:v>
       </x:c>
-      <x:c r="O75" s="72" t="str"/>
-      <x:c r="P75" s="72" t="str"/>
+      <x:c r="O75" s="72"/>
+      <x:c r="P75" s="72"/>
       <x:c r="Q75" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4547,7 +4564,7 @@
       <x:c r="G76" s="76" t="str">
         <x:v>ogden-nature-center.jpg</x:v>
       </x:c>
-      <x:c r="H76" s="76" t="str"/>
+      <x:c r="H76" s="76"/>
       <x:c r="I76" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4566,8 +4583,8 @@
       <x:c r="N76" s="76" t="str">
         <x:v>https://ogdennaturecenter.org/</x:v>
       </x:c>
-      <x:c r="O76" s="76" t="str"/>
-      <x:c r="P76" s="76" t="str"/>
+      <x:c r="O76" s="76"/>
+      <x:c r="P76" s="76"/>
       <x:c r="Q76" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4594,7 +4611,7 @@
       <x:c r="G77" s="72" t="str">
         <x:v>25th-street-historic-district.jpg</x:v>
       </x:c>
-      <x:c r="H77" s="72" t="str"/>
+      <x:c r="H77" s="72"/>
       <x:c r="I77" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4613,8 +4630,8 @@
       <x:c r="N77" s="72" t="str">
         <x:v>https://www.visitogden.com/</x:v>
       </x:c>
-      <x:c r="O77" s="72" t="str"/>
-      <x:c r="P77" s="72" t="str"/>
+      <x:c r="O77" s="72"/>
+      <x:c r="P77" s="72"/>
       <x:c r="Q77" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4641,7 +4658,7 @@
       <x:c r="G78" s="76" t="str">
         <x:v>hill-aerospace-museum.jpg</x:v>
       </x:c>
-      <x:c r="H78" s="76" t="str"/>
+      <x:c r="H78" s="76"/>
       <x:c r="I78" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4660,8 +4677,8 @@
       <x:c r="N78" s="76" t="str">
         <x:v>https://www.aerospaceutah.com/</x:v>
       </x:c>
-      <x:c r="O78" s="76" t="str"/>
-      <x:c r="P78" s="76" t="str"/>
+      <x:c r="O78" s="76"/>
+      <x:c r="P78" s="76"/>
       <x:c r="Q78" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4688,7 +4705,7 @@
       <x:c r="G79" s="72" t="str">
         <x:v>salomon-center.jpg</x:v>
       </x:c>
-      <x:c r="H79" s="72" t="str"/>
+      <x:c r="H79" s="72"/>
       <x:c r="I79" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4707,8 +4724,8 @@
       <x:c r="N79" s="72" t="str">
         <x:v>https://www.visitogden.com/</x:v>
       </x:c>
-      <x:c r="O79" s="72" t="str"/>
-      <x:c r="P79" s="72" t="str"/>
+      <x:c r="O79" s="72"/>
+      <x:c r="P79" s="72"/>
       <x:c r="Q79" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4735,7 +4752,7 @@
       <x:c r="G80" s="76" t="str">
         <x:v>weber-state-university.jpg</x:v>
       </x:c>
-      <x:c r="H80" s="76" t="str"/>
+      <x:c r="H80" s="76"/>
       <x:c r="I80" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4754,8 +4771,8 @@
       <x:c r="N80" s="76" t="str">
         <x:v>https://www.weber.edu/</x:v>
       </x:c>
-      <x:c r="O80" s="76" t="str"/>
-      <x:c r="P80" s="76" t="str"/>
+      <x:c r="O80" s="76"/>
+      <x:c r="P80" s="76"/>
       <x:c r="Q80" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4782,7 +4799,7 @@
       <x:c r="G81" s="72" t="str">
         <x:v>ogden-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H81" s="72" t="str"/>
+      <x:c r="H81" s="72"/>
       <x:c r="I81" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4801,8 +4818,8 @@
       <x:c r="N81" s="72" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O81" s="72" t="str"/>
-      <x:c r="P81" s="72" t="str"/>
+      <x:c r="O81" s="72"/>
+      <x:c r="P81" s="72"/>
       <x:c r="Q81" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4829,7 +4846,7 @@
       <x:c r="G82" s="76" t="str">
         <x:v>pineview-reservoir.jpg</x:v>
       </x:c>
-      <x:c r="H82" s="76" t="str"/>
+      <x:c r="H82" s="76"/>
       <x:c r="I82" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4848,8 +4865,8 @@
       <x:c r="N82" s="76" t="str">
         <x:v>https://www.visitogden.com/</x:v>
       </x:c>
-      <x:c r="O82" s="76" t="str"/>
-      <x:c r="P82" s="76" t="str"/>
+      <x:c r="O82" s="76"/>
+      <x:c r="P82" s="76"/>
       <x:c r="Q82" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4876,7 +4893,7 @@
       <x:c r="G83" s="72" t="str">
         <x:v>fielding-garr-ranch.jpg</x:v>
       </x:c>
-      <x:c r="H83" s="72" t="str"/>
+      <x:c r="H83" s="72"/>
       <x:c r="I83" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4895,8 +4912,8 @@
       <x:c r="N83" s="72" t="str">
         <x:v>https://stateparks.utah.gov/parks/antelope-island/</x:v>
       </x:c>
-      <x:c r="O83" s="72" t="str"/>
-      <x:c r="P83" s="72" t="str"/>
+      <x:c r="O83" s="72"/>
+      <x:c r="P83" s="72"/>
       <x:c r="Q83" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4923,7 +4940,7 @@
       <x:c r="G84" s="76" t="str">
         <x:v>saltair.jpg</x:v>
       </x:c>
-      <x:c r="H84" s="76" t="str"/>
+      <x:c r="H84" s="76"/>
       <x:c r="I84" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4942,8 +4959,8 @@
       <x:c r="N84" s="76" t="str">
         <x:v>https://saltairutah.com/</x:v>
       </x:c>
-      <x:c r="O84" s="76" t="str"/>
-      <x:c r="P84" s="76" t="str"/>
+      <x:c r="O84" s="76"/>
+      <x:c r="P84" s="76"/>
       <x:c r="Q84" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4970,7 +4987,7 @@
       <x:c r="G85" s="72" t="str">
         <x:v>spiral-jetty.jpg</x:v>
       </x:c>
-      <x:c r="H85" s="72" t="str"/>
+      <x:c r="H85" s="72"/>
       <x:c r="I85" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -4989,8 +5006,8 @@
       <x:c r="N85" s="72" t="str">
         <x:v>https://www.utah.com/</x:v>
       </x:c>
-      <x:c r="O85" s="72" t="str"/>
-      <x:c r="P85" s="72" t="str"/>
+      <x:c r="O85" s="72"/>
+      <x:c r="P85" s="72"/>
       <x:c r="Q85" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5017,7 +5034,7 @@
       <x:c r="G86" s="76" t="str">
         <x:v>bonneville-salt-flats.jpg</x:v>
       </x:c>
-      <x:c r="H86" s="76" t="str"/>
+      <x:c r="H86" s="76"/>
       <x:c r="I86" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5036,8 +5053,8 @@
       <x:c r="N86" s="76" t="str">
         <x:v>https://stateparks.utah.gov/</x:v>
       </x:c>
-      <x:c r="O86" s="76" t="str"/>
-      <x:c r="P86" s="76" t="str"/>
+      <x:c r="O86" s="76"/>
+      <x:c r="P86" s="76"/>
       <x:c r="Q86" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5064,7 +5081,7 @@
       <x:c r="G87" s="72" t="str">
         <x:v>farmington-bay.jpg</x:v>
       </x:c>
-      <x:c r="H87" s="72" t="str"/>
+      <x:c r="H87" s="72"/>
       <x:c r="I87" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5083,8 +5100,8 @@
       <x:c r="N87" s="72" t="str">
         <x:v>https://www.visitutah.com/</x:v>
       </x:c>
-      <x:c r="O87" s="72" t="str"/>
-      <x:c r="P87" s="72" t="str"/>
+      <x:c r="O87" s="72"/>
+      <x:c r="P87" s="72"/>
       <x:c r="Q87" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5111,7 +5128,7 @@
       <x:c r="G88" s="76" t="str">
         <x:v>bountiful.jpg</x:v>
       </x:c>
-      <x:c r="H88" s="76" t="str"/>
+      <x:c r="H88" s="76"/>
       <x:c r="I88" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5130,8 +5147,8 @@
       <x:c r="N88" s="76" t="str">
         <x:v>https://www.visitutah.com/</x:v>
       </x:c>
-      <x:c r="O88" s="76" t="str"/>
-      <x:c r="P88" s="76" t="str"/>
+      <x:c r="O88" s="76"/>
+      <x:c r="P88" s="76"/>
       <x:c r="Q88" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5158,7 +5175,7 @@
       <x:c r="G89" s="72" t="str">
         <x:v>kaysville.jpg</x:v>
       </x:c>
-      <x:c r="H89" s="72" t="str"/>
+      <x:c r="H89" s="72"/>
       <x:c r="I89" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5177,8 +5194,8 @@
       <x:c r="N89" s="72" t="str">
         <x:v>https://www.visitutah.com/</x:v>
       </x:c>
-      <x:c r="O89" s="72" t="str"/>
-      <x:c r="P89" s="72" t="str"/>
+      <x:c r="O89" s="72"/>
+      <x:c r="P89" s="72"/>
       <x:c r="Q89" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5205,7 +5222,7 @@
       <x:c r="G90" s="76" t="str">
         <x:v>layton.jpg</x:v>
       </x:c>
-      <x:c r="H90" s="76" t="str"/>
+      <x:c r="H90" s="76"/>
       <x:c r="I90" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5224,8 +5241,8 @@
       <x:c r="N90" s="76" t="str">
         <x:v>https://www.visitutah.com/</x:v>
       </x:c>
-      <x:c r="O90" s="76" t="str"/>
-      <x:c r="P90" s="76" t="str"/>
+      <x:c r="O90" s="76"/>
+      <x:c r="P90" s="76"/>
       <x:c r="Q90" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5252,7 +5269,7 @@
       <x:c r="G91" s="72" t="str">
         <x:v>station-park-farmington.jpg</x:v>
       </x:c>
-      <x:c r="H91" s="72" t="str"/>
+      <x:c r="H91" s="72"/>
       <x:c r="I91" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5271,8 +5288,8 @@
       <x:c r="N91" s="72" t="str">
         <x:v>https://www.stationpark.com/</x:v>
       </x:c>
-      <x:c r="O91" s="72" t="str"/>
-      <x:c r="P91" s="72" t="str"/>
+      <x:c r="O91" s="72"/>
+      <x:c r="P91" s="72"/>
       <x:c r="Q91" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5299,7 +5316,7 @@
       <x:c r="G92" s="76" t="str">
         <x:v>city-creek-center.jpg</x:v>
       </x:c>
-      <x:c r="H92" s="76" t="str"/>
+      <x:c r="H92" s="76"/>
       <x:c r="I92" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5318,8 +5335,8 @@
       <x:c r="N92" s="76" t="str">
         <x:v>https://www.shopcitycreekcenter.com/</x:v>
       </x:c>
-      <x:c r="O92" s="76" t="str"/>
-      <x:c r="P92" s="76" t="str"/>
+      <x:c r="O92" s="76"/>
+      <x:c r="P92" s="76"/>
       <x:c r="Q92" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5346,7 +5363,7 @@
       <x:c r="G93" s="72" t="str">
         <x:v>trolley-square.jpg</x:v>
       </x:c>
-      <x:c r="H93" s="72" t="str"/>
+      <x:c r="H93" s="72"/>
       <x:c r="I93" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5365,8 +5382,8 @@
       <x:c r="N93" s="72" t="str">
         <x:v>https://www.trolleysquare.com/</x:v>
       </x:c>
-      <x:c r="O93" s="72" t="str"/>
-      <x:c r="P93" s="72" t="str"/>
+      <x:c r="O93" s="72"/>
+      <x:c r="P93" s="72"/>
       <x:c r="Q93" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5393,7 +5410,7 @@
       <x:c r="G94" s="76" t="str">
         <x:v>900-south-historic-district.jpg</x:v>
       </x:c>
-      <x:c r="H94" s="76" t="str"/>
+      <x:c r="H94" s="76"/>
       <x:c r="I94" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5412,8 +5429,8 @@
       <x:c r="N94" s="76" t="str">
         <x:v>https://www.slc.gov/</x:v>
       </x:c>
-      <x:c r="O94" s="76" t="str"/>
-      <x:c r="P94" s="76" t="str"/>
+      <x:c r="O94" s="76"/>
+      <x:c r="P94" s="76"/>
       <x:c r="Q94" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5440,7 +5457,7 @@
       <x:c r="G95" s="72" t="str">
         <x:v>sugar-house.jpg</x:v>
       </x:c>
-      <x:c r="H95" s="72" t="str"/>
+      <x:c r="H95" s="72"/>
       <x:c r="I95" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5459,8 +5476,8 @@
       <x:c r="N95" s="72" t="str">
         <x:v>https://www.slc.gov/</x:v>
       </x:c>
-      <x:c r="O95" s="72" t="str"/>
-      <x:c r="P95" s="72" t="str"/>
+      <x:c r="O95" s="72"/>
+      <x:c r="P95" s="72"/>
       <x:c r="Q95" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5487,7 +5504,7 @@
       <x:c r="G96" s="76" t="str">
         <x:v>holladay.jpg</x:v>
       </x:c>
-      <x:c r="H96" s="76" t="str"/>
+      <x:c r="H96" s="76"/>
       <x:c r="I96" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5506,8 +5523,8 @@
       <x:c r="N96" s="76" t="str">
         <x:v>https://www.holladayut.gov/</x:v>
       </x:c>
-      <x:c r="O96" s="76" t="str"/>
-      <x:c r="P96" s="76" t="str"/>
+      <x:c r="O96" s="76"/>
+      <x:c r="P96" s="76"/>
       <x:c r="Q96" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5534,7 +5551,7 @@
       <x:c r="G97" s="72" t="str">
         <x:v>draper.jpg</x:v>
       </x:c>
-      <x:c r="H97" s="72" t="str"/>
+      <x:c r="H97" s="72"/>
       <x:c r="I97" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5553,8 +5570,8 @@
       <x:c r="N97" s="72" t="str">
         <x:v>https://www.draperutah.gov/</x:v>
       </x:c>
-      <x:c r="O97" s="72" t="str"/>
-      <x:c r="P97" s="72" t="str"/>
+      <x:c r="O97" s="72"/>
+      <x:c r="P97" s="72"/>
       <x:c r="Q97" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5581,7 +5598,7 @@
       <x:c r="G98" s="76" t="str">
         <x:v>sandy.jpg</x:v>
       </x:c>
-      <x:c r="H98" s="76" t="str"/>
+      <x:c r="H98" s="76"/>
       <x:c r="I98" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5600,8 +5617,8 @@
       <x:c r="N98" s="76" t="str">
         <x:v>https://www.sandy.utah.gov/</x:v>
       </x:c>
-      <x:c r="O98" s="76" t="str"/>
-      <x:c r="P98" s="76" t="str"/>
+      <x:c r="O98" s="76"/>
+      <x:c r="P98" s="76"/>
       <x:c r="Q98" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5628,7 +5645,7 @@
       <x:c r="G99" s="72" t="str">
         <x:v>mountain-dell-reservoir.jpg</x:v>
       </x:c>
-      <x:c r="H99" s="72" t="str"/>
+      <x:c r="H99" s="72"/>
       <x:c r="I99" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5647,8 +5664,8 @@
       <x:c r="N99" s="72" t="str">
         <x:v>https://www.slc.gov/parks/</x:v>
       </x:c>
-      <x:c r="O99" s="72" t="str"/>
-      <x:c r="P99" s="72" t="str"/>
+      <x:c r="O99" s="72"/>
+      <x:c r="P99" s="72"/>
       <x:c r="Q99" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5675,7 +5692,7 @@
       <x:c r="G100" s="76" t="str">
         <x:v>emigration-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H100" s="76" t="str"/>
+      <x:c r="H100" s="76"/>
       <x:c r="I100" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5694,8 +5711,8 @@
       <x:c r="N100" s="76" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O100" s="76" t="str"/>
-      <x:c r="P100" s="76" t="str"/>
+      <x:c r="O100" s="76"/>
+      <x:c r="P100" s="76"/>
       <x:c r="Q100" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5722,7 +5739,7 @@
       <x:c r="G101" s="72" t="str">
         <x:v>thanksgiving-point.jpg</x:v>
       </x:c>
-      <x:c r="H101" s="72" t="str"/>
+      <x:c r="H101" s="72"/>
       <x:c r="I101" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5741,8 +5758,8 @@
       <x:c r="N101" s="72" t="str">
         <x:v>https://www.thanksgivingpoint.org/</x:v>
       </x:c>
-      <x:c r="O101" s="72" t="str"/>
-      <x:c r="P101" s="72" t="str"/>
+      <x:c r="O101" s="72"/>
+      <x:c r="P101" s="72"/>
       <x:c r="Q101" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5769,7 +5786,7 @@
       <x:c r="G102" s="76" t="str">
         <x:v>loveland-living-planet-aquarium.jpg</x:v>
       </x:c>
-      <x:c r="H102" s="76" t="str"/>
+      <x:c r="H102" s="76"/>
       <x:c r="I102" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5788,8 +5805,8 @@
       <x:c r="N102" s="76" t="str">
         <x:v>https://livingplanetaquarium.org/</x:v>
       </x:c>
-      <x:c r="O102" s="76" t="str"/>
-      <x:c r="P102" s="76" t="str"/>
+      <x:c r="O102" s="76"/>
+      <x:c r="P102" s="76"/>
       <x:c r="Q102" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5816,7 +5833,7 @@
       <x:c r="G103" s="72" t="str">
         <x:v>provo.jpg</x:v>
       </x:c>
-      <x:c r="H103" s="72" t="str"/>
+      <x:c r="H103" s="72"/>
       <x:c r="I103" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5835,8 +5852,8 @@
       <x:c r="N103" s="72" t="str">
         <x:v>https://www.provo.org/</x:v>
       </x:c>
-      <x:c r="O103" s="72" t="str"/>
-      <x:c r="P103" s="72" t="str"/>
+      <x:c r="O103" s="72"/>
+      <x:c r="P103" s="72"/>
       <x:c r="Q103" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5863,7 +5880,7 @@
       <x:c r="G104" s="76" t="str">
         <x:v>brigham-young-university.jpg</x:v>
       </x:c>
-      <x:c r="H104" s="76" t="str"/>
+      <x:c r="H104" s="76"/>
       <x:c r="I104" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
@@ -5882,8 +5899,8 @@
       <x:c r="N104" s="76" t="str">
         <x:v>https://www.byu.edu/</x:v>
       </x:c>
-      <x:c r="O104" s="76" t="str"/>
-      <x:c r="P104" s="76" t="str"/>
+      <x:c r="O104" s="76"/>
+      <x:c r="P104" s="76"/>
       <x:c r="Q104" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>

</xml_diff>

<commit_message>
Refresh Around You place imagery
</commit_message>
<xml_diff>
--- a/assets-source/passenger/around-you/around-you-image-inventory.xlsx
+++ b/assets-source/passenger/around-you/around-you-image-inventory.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R5244dc85ab4e44c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="Rc49bc1cb6233491d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4a7060fa3f29475e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="R3e0fa0629b684141"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -727,7 +727,6 @@
         <x:v>Total places</x:v>
       </x:c>
       <x:c r="B11" s="33" t="n">
-        <x:f>COUNTA('Inventory'!A5:A104)</x:f>
         <x:v>100</x:v>
       </x:c>
       <x:c r="C11" s="28"/>
@@ -742,7 +741,6 @@
         <x:v>Active in app</x:v>
       </x:c>
       <x:c r="B12" s="33" t="n">
-        <x:f>COUNTIF('Inventory'!F5:F104,"Active in app")</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="C12" s="28"/>
@@ -757,7 +755,6 @@
         <x:v>Candidates — not active</x:v>
       </x:c>
       <x:c r="B13" s="33" t="n">
-        <x:f>COUNTIF('Inventory'!F5:F104,"Candidate — not active")</x:f>
         <x:v>68</x:v>
       </x:c>
       <x:c r="C13" s="28"/>
@@ -1114,7 +1111,7 @@
       <x:c r="J5" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K5" s="72" t="n">
+      <x:c r="K5" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L5" s="72" t="str">
@@ -1123,7 +1120,7 @@
       <x:c r="M5" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N5" s="72"/>
+      <x:c r="N5" s="72" t="str"/>
       <x:c r="O5" s="72" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1165,7 +1162,7 @@
       <x:c r="J6" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K6" s="76" t="n">
+      <x:c r="K6" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L6" s="76" t="str">
@@ -1174,7 +1171,7 @@
       <x:c r="M6" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N6" s="76"/>
+      <x:c r="N6" s="76" t="str"/>
       <x:c r="O6" s="76" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1216,7 +1213,7 @@
       <x:c r="J7" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K7" s="72" t="n">
+      <x:c r="K7" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L7" s="72" t="str">
@@ -1225,7 +1222,7 @@
       <x:c r="M7" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N7" s="72"/>
+      <x:c r="N7" s="72" t="str"/>
       <x:c r="O7" s="72" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1259,7 +1256,7 @@
         <x:v>utah-state-capitol.jpg</x:v>
       </x:c>
       <x:c r="H8" s="76" t="str">
-        <x:v>/images/passenger/around-you/user/utah-state-capitol-juan.webp</x:v>
+        <x:v>/images/passenger/around-you/user/utah-state-capitol-night-gardens-juan.webp</x:v>
       </x:c>
       <x:c r="I8" s="74" t="str">
         <x:v>Own local asset</x:v>
@@ -1267,7 +1264,7 @@
       <x:c r="J8" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K8" s="76" t="n">
+      <x:c r="K8" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L8" s="76" t="str">
@@ -1284,7 +1281,7 @@
         <x:v>User-owned original; permission confirmed</x:v>
       </x:c>
       <x:c r="Q8" s="76" t="str">
-        <x:v>Selected from renamed utah-state-capitol-night-gardens.jpeg; user-owned hero showing the Capitol grounds and dome, optimized to local WebP with metadata stripped.</x:v>
+        <x:v>Selected from user-photos/utah-state-capitol-night-gardens.jpeg; user-owned night garden hero with the illuminated dome and grounds, optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -1310,7 +1307,7 @@
         <x:v>temple-square.jpg</x:v>
       </x:c>
       <x:c r="H9" s="72" t="str">
-        <x:v>/images/passenger/around-you/user/temple-square-juan.webp</x:v>
+        <x:v>/images/passenger/around-you/user/temple-square-spires-juan.webp</x:v>
       </x:c>
       <x:c r="I9" s="74" t="str">
         <x:v>Own local asset</x:v>
@@ -1318,7 +1315,7 @@
       <x:c r="J9" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K9" s="72" t="n">
+      <x:c r="K9" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L9" s="72" t="str">
@@ -1335,7 +1332,7 @@
         <x:v>User-owned original; permission confirmed</x:v>
       </x:c>
       <x:c r="Q9" s="72" t="str">
-        <x:v>Selected from renamed temple-square-night.jpeg; user-owned hero showing Temple Square architecture, optimized to local WebP with metadata stripped.</x:v>
+        <x:v>Selected from user-photos/temple-square-spires.jpeg; daylight hero showing Temple Square spires, architecture and grounds, optimized to local WebP with metadata stripped.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
@@ -1369,7 +1366,7 @@
       <x:c r="J10" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K10" s="76" t="n">
+      <x:c r="K10" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L10" s="76" t="str">
@@ -1378,7 +1375,7 @@
       <x:c r="M10" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N10" s="76"/>
+      <x:c r="N10" s="76" t="str"/>
       <x:c r="O10" s="76" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1420,7 +1417,7 @@
       <x:c r="J11" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K11" s="72" t="n">
+      <x:c r="K11" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L11" s="72" t="str">
@@ -1429,7 +1426,7 @@
       <x:c r="M11" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N11" s="72"/>
+      <x:c r="N11" s="72" t="str"/>
       <x:c r="O11" s="72" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1463,7 +1460,7 @@
         <x:v>university-of-utah.jpg</x:v>
       </x:c>
       <x:c r="H12" s="76" t="str">
-        <x:v>/images/passenger/around-you/curated/university-of-utah-campus.webp</x:v>
+        <x:v>/images/passenger/around-you/curated/university-of-utah-presidents-circle.webp</x:v>
       </x:c>
       <x:c r="I12" s="77" t="str">
         <x:v>Curated Commons asset</x:v>
@@ -1471,7 +1468,7 @@
       <x:c r="J12" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K12" s="76" t="n">
+      <x:c r="K12" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L12" s="76" t="str">
@@ -1490,7 +1487,7 @@
         <x:v>CC BY-SA 4.0 — attribution and share-alike required</x:v>
       </x:c>
       <x:c r="Q12" s="76" t="str">
-        <x:v>Curated from utah-presidents-circle.jpg; cropped and optimized to metadata-free WebP with the campus architecture clearly visible.</x:v>
+        <x:v>Refreshed with a wide Presidents Circle campus view and Wasatch context; cropped and optimized to metadata-free WebP.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -1516,7 +1513,7 @@
         <x:v>red-butte-garden.jpg</x:v>
       </x:c>
       <x:c r="H13" s="72" t="str">
-        <x:v>/images/passenger/around-you/curated/red-butte-garden.webp</x:v>
+        <x:v>/images/passenger/around-you/curated/red-butte-garden-orangerie.webp</x:v>
       </x:c>
       <x:c r="I13" s="77" t="str">
         <x:v>Curated Commons asset</x:v>
@@ -1524,7 +1521,7 @@
       <x:c r="J13" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K13" s="72" t="n">
+      <x:c r="K13" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L13" s="72" t="str">
@@ -1534,16 +1531,16 @@
         <x:v>Active coordinates</x:v>
       </x:c>
       <x:c r="N13" s="72" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:Red_Butte_Garden2.jpg</x:v>
+        <x:v>https://commons.wikimedia.org/wiki/File:Orangerie_-_Red_Butte_Garden_and_Arboretum_-_DSC07479.JPG</x:v>
       </x:c>
       <x:c r="O13" s="72" t="str">
-        <x:v>Wikimedia Commons — C.Maylett</x:v>
+        <x:v>Wikimedia Commons — Daderot</x:v>
       </x:c>
       <x:c r="P13" s="72" t="str">
-        <x:v>CC BY-SA 3.0 — attribution and share-alike required</x:v>
+        <x:v>CC0 / public domain</x:v>
       </x:c>
       <x:c r="Q13" s="72" t="str">
-        <x:v>Curated garden interior image; optimized to local WebP with metadata stripped.</x:v>
+        <x:v>Refreshed with an attractive Red Butte Garden Orangerie interior; cropped and optimized to metadata-free WebP.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
@@ -1568,14 +1565,14 @@
       <x:c r="G14" s="76" t="str">
         <x:v>this-is-the-place.jpg</x:v>
       </x:c>
-      <x:c r="H14" s="76"/>
+      <x:c r="H14" s="76" t="str"/>
       <x:c r="I14" s="77" t="str">
         <x:v>Original staged — rights recorded</x:v>
       </x:c>
       <x:c r="J14" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K14" s="76" t="n">
+      <x:c r="K14" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L14" s="76" t="str">
@@ -1602,10 +1599,10 @@
         <x:v>salt-lake-city-airport</x:v>
       </x:c>
       <x:c r="B15" s="72" t="str">
-        <x:v>salt lake city airport</x:v>
+        <x:v>Salt Lake City International Airport</x:v>
       </x:c>
       <x:c r="C15" s="72" t="str">
-        <x:v>salt lake city airport</x:v>
+        <x:v>Aeropuerto Internacional de Salt Lake City</x:v>
       </x:c>
       <x:c r="D15" s="72" t="str">
         <x:v>transportation</x:v>
@@ -1620,7 +1617,7 @@
         <x:v>salt-lake-city-airport.jpg</x:v>
       </x:c>
       <x:c r="H15" s="72" t="str">
-        <x:v>/images/passenger/around-you/curated/salt-lake-city-airport-terminal.webp</x:v>
+        <x:v>/images/passenger/around-you/curated/salt-lake-city-airport-concourse-b.webp</x:v>
       </x:c>
       <x:c r="I15" s="77" t="str">
         <x:v>Curated Commons asset</x:v>
@@ -1628,7 +1625,7 @@
       <x:c r="J15" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K15" s="72" t="n">
+      <x:c r="K15" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L15" s="72" t="str">
@@ -1638,16 +1635,16 @@
         <x:v>Active coordinates</x:v>
       </x:c>
       <x:c r="N15" s="72" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:2015-04-14_00_11_43_View_towards_the_International_Terminal_and_Concourse_D_from_the_inner_end_of_Concourse_C_in_Salt_Lake_City_International_Airport,_Utah.jpg</x:v>
+        <x:v>https://commons.wikimedia.org/wiki/File:KSLC_Concourse_B_interior.jpg</x:v>
       </x:c>
       <x:c r="O15" s="72" t="str">
-        <x:v>Wikimedia Commons — Famartin</x:v>
+        <x:v>Wikimedia Commons — ECTran71</x:v>
       </x:c>
       <x:c r="P15" s="72" t="str">
         <x:v>CC BY-SA 4.0 — attribution and share-alike required</x:v>
       </x:c>
       <x:c r="Q15" s="72" t="str">
-        <x:v>Curated terminal/interior view rather than an aerial; optimized to local WebP with metadata stripped.</x:v>
+        <x:v>Refreshed with a bright SLC Concourse B interior and recognizable terminal context; optimized to metadata-free WebP.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
@@ -1681,7 +1678,7 @@
       <x:c r="J16" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K16" s="76" t="n">
+      <x:c r="K16" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L16" s="76" t="str">
@@ -1690,7 +1687,7 @@
       <x:c r="M16" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N16" s="76"/>
+      <x:c r="N16" s="76" t="str"/>
       <x:c r="O16" s="76" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1723,14 +1720,14 @@
       <x:c r="G17" s="72" t="str">
         <x:v>parleys-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H17" s="72"/>
+      <x:c r="H17" s="72" t="str"/>
       <x:c r="I17" s="77" t="str">
         <x:v>Original staged — rights recorded</x:v>
       </x:c>
       <x:c r="J17" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K17" s="72" t="n">
+      <x:c r="K17" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L17" s="72" t="str">
@@ -1757,10 +1754,10 @@
         <x:v>lagoon-amusement-park</x:v>
       </x:c>
       <x:c r="B18" s="76" t="str">
-        <x:v>Lagoon</x:v>
+        <x:v>Lagoon Amusement Park</x:v>
       </x:c>
       <x:c r="C18" s="76" t="str">
-        <x:v>Lagoon</x:v>
+        <x:v>Parque de Atracciones Lagoon</x:v>
       </x:c>
       <x:c r="D18" s="76" t="str">
         <x:v>culture</x:v>
@@ -1775,7 +1772,7 @@
         <x:v>lagoon-amusement-park.jpg</x:v>
       </x:c>
       <x:c r="H18" s="76" t="str">
-        <x:v>/images/passenger/around-you/curated/lagoon-exterior.webp</x:v>
+        <x:v>/images/passenger/around-you/curated/lagoon-entrance.webp</x:v>
       </x:c>
       <x:c r="I18" s="74" t="str">
         <x:v>Curated Commons asset</x:v>
@@ -1783,7 +1780,7 @@
       <x:c r="J18" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K18" s="76" t="n">
+      <x:c r="K18" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L18" s="76" t="str">
@@ -1793,16 +1790,16 @@
         <x:v>Active coordinates</x:v>
       </x:c>
       <x:c r="N18" s="76" t="str">
-        <x:v>https://commons.wikimedia.org/wiki/File:Lagoon_Roller_Coaster_winter.jpeg</x:v>
+        <x:v>https://commons.wikimedia.org/wiki/File:Lagoon_sign_(43886157261).jpg</x:v>
       </x:c>
       <x:c r="O18" s="76" t="str">
-        <x:v>Wikimedia Commons — Ntsimp</x:v>
+        <x:v>Wikimedia Commons — Ben P L</x:v>
       </x:c>
       <x:c r="P18" s="76" t="str">
-        <x:v>CC0 — no attribution required</x:v>
+        <x:v>CC BY-SA 2.0 — attribution and share-alike required</x:v>
       </x:c>
       <x:c r="Q18" s="76" t="str">
-        <x:v>Curated exterior attraction view; optimized to local WebP with metadata stripped.</x:v>
+        <x:v>Refreshed with a recognizable Lagoon entrance/sign view from outside the park; cropped and optimized to metadata-free WebP.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
@@ -1827,14 +1824,14 @@
       <x:c r="G19" s="72" t="str">
         <x:v>ogden.jpg</x:v>
       </x:c>
-      <x:c r="H19" s="72"/>
+      <x:c r="H19" s="72" t="str"/>
       <x:c r="I19" s="77" t="str">
         <x:v>Original staged — rights recorded</x:v>
       </x:c>
       <x:c r="J19" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K19" s="72" t="n">
+      <x:c r="K19" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L19" s="72" t="str">
@@ -1887,7 +1884,7 @@
       <x:c r="J20" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K20" s="76" t="n">
+      <x:c r="K20" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L20" s="76" t="str">
@@ -1896,7 +1893,7 @@
       <x:c r="M20" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N20" s="76"/>
+      <x:c r="N20" s="76" t="str"/>
       <x:c r="O20" s="76" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1938,7 +1935,7 @@
       <x:c r="J21" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K21" s="72" t="n">
+      <x:c r="K21" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L21" s="72" t="str">
@@ -1947,7 +1944,7 @@
       <x:c r="M21" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N21" s="72"/>
+      <x:c r="N21" s="72" t="str"/>
       <x:c r="O21" s="72" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -1989,7 +1986,7 @@
       <x:c r="J22" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K22" s="76" t="n">
+      <x:c r="K22" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L22" s="76" t="str">
@@ -1998,7 +1995,7 @@
       <x:c r="M22" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N22" s="76"/>
+      <x:c r="N22" s="76" t="str"/>
       <x:c r="O22" s="76" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -2040,7 +2037,7 @@
       <x:c r="J23" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K23" s="72" t="n">
+      <x:c r="K23" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L23" s="72" t="str">
@@ -2049,7 +2046,7 @@
       <x:c r="M23" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N23" s="72"/>
+      <x:c r="N23" s="72" t="str"/>
       <x:c r="O23" s="72" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -2083,7 +2080,7 @@
         <x:v>kimball-junction.jpg</x:v>
       </x:c>
       <x:c r="H24" s="76" t="str">
-        <x:v>/images/passenger/around-you/curated/kimball-junction-sunset.webp</x:v>
+        <x:v>/images/passenger/around-you/curated/kimball-junction-scenic.webp</x:v>
       </x:c>
       <x:c r="I24" s="74" t="str">
         <x:v>Curated Commons asset</x:v>
@@ -2091,7 +2088,7 @@
       <x:c r="J24" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K24" s="76" t="n">
+      <x:c r="K24" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L24" s="76" t="str">
@@ -2107,10 +2104,10 @@
         <x:v>Wikimedia Commons — Patrick Hendry</x:v>
       </x:c>
       <x:c r="P24" s="76" t="str">
-        <x:v>CC0 — no attribution required</x:v>
+        <x:v>CC0 / public domain</x:v>
       </x:c>
       <x:c r="Q24" s="76" t="str">
-        <x:v>Curated sunset view for the Kimball Junction corridor; optimized to local WebP with metadata stripped.</x:v>
+        <x:v>Replaced the bus/transit view with a scenic Kimball Junction mountain gateway; cropped and optimized to metadata-free WebP.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
@@ -2144,7 +2141,7 @@
       <x:c r="J25" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K25" s="72" t="n">
+      <x:c r="K25" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L25" s="72" t="str">
@@ -2153,7 +2150,7 @@
       <x:c r="M25" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N25" s="72"/>
+      <x:c r="N25" s="72" t="str"/>
       <x:c r="O25" s="72" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -2195,7 +2192,7 @@
       <x:c r="J26" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K26" s="76" t="n">
+      <x:c r="K26" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L26" s="76" t="str">
@@ -2207,8 +2204,8 @@
       <x:c r="N26" s="76" t="str">
         <x:v>https://nhmu.utah.edu/</x:v>
       </x:c>
-      <x:c r="O26" s="76"/>
-      <x:c r="P26" s="76"/>
+      <x:c r="O26" s="76" t="str"/>
+      <x:c r="P26" s="76" t="str"/>
       <x:c r="Q26" s="76" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2244,7 +2241,7 @@
       <x:c r="J27" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K27" s="72" t="n">
+      <x:c r="K27" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L27" s="72" t="str">
@@ -2256,8 +2253,8 @@
       <x:c r="N27" s="72" t="str">
         <x:v>https://www.slc.gov/parks/parks-division/ensign-peak-nature-park/</x:v>
       </x:c>
-      <x:c r="O27" s="72"/>
-      <x:c r="P27" s="72"/>
+      <x:c r="O27" s="72" t="str"/>
+      <x:c r="P27" s="72" t="str"/>
       <x:c r="Q27" s="72" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2293,7 +2290,7 @@
       <x:c r="J28" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K28" s="76" t="n">
+      <x:c r="K28" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L28" s="76" t="str">
@@ -2305,8 +2302,8 @@
       <x:c r="N28" s="76" t="str">
         <x:v>https://tracyaviary.org/</x:v>
       </x:c>
-      <x:c r="O28" s="76"/>
-      <x:c r="P28" s="76"/>
+      <x:c r="O28" s="76" t="str"/>
+      <x:c r="P28" s="76" t="str"/>
       <x:c r="Q28" s="76" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2342,7 +2339,7 @@
       <x:c r="J29" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K29" s="72" t="n">
+      <x:c r="K29" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L29" s="72" t="str">
@@ -2354,8 +2351,8 @@
       <x:c r="N29" s="72" t="str">
         <x:v>https://www.hoglezoo.org/</x:v>
       </x:c>
-      <x:c r="O29" s="72"/>
-      <x:c r="P29" s="72"/>
+      <x:c r="O29" s="72" t="str"/>
+      <x:c r="P29" s="72" t="str"/>
       <x:c r="Q29" s="72" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2391,7 +2388,7 @@
       <x:c r="J30" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K30" s="76" t="n">
+      <x:c r="K30" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L30" s="76" t="str">
@@ -2400,7 +2397,7 @@
       <x:c r="M30" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N30" s="76"/>
+      <x:c r="N30" s="76" t="str"/>
       <x:c r="O30" s="76" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -2442,7 +2439,7 @@
       <x:c r="J31" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K31" s="72" t="n">
+      <x:c r="K31" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L31" s="72" t="str">
@@ -2454,8 +2451,8 @@
       <x:c r="N31" s="72" t="str">
         <x:v>https://www.slc.gov/parks/parks-division/gilgal-sculpture-garden/</x:v>
       </x:c>
-      <x:c r="O31" s="72"/>
-      <x:c r="P31" s="72"/>
+      <x:c r="O31" s="72" t="str"/>
+      <x:c r="P31" s="72" t="str"/>
       <x:c r="Q31" s="72" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2491,7 +2488,7 @@
       <x:c r="J32" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K32" s="76" t="n">
+      <x:c r="K32" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L32" s="76" t="str">
@@ -2500,7 +2497,7 @@
       <x:c r="M32" s="76" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N32" s="76"/>
+      <x:c r="N32" s="76" t="str"/>
       <x:c r="O32" s="76" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -2542,7 +2539,7 @@
       <x:c r="J33" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K33" s="72" t="n">
+      <x:c r="K33" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L33" s="72" t="str">
@@ -2554,8 +2551,8 @@
       <x:c r="N33" s="72" t="str">
         <x:v>https://www.parkcity.org/departments/trails-open-space/historic-mcpolin-barn</x:v>
       </x:c>
-      <x:c r="O33" s="72"/>
-      <x:c r="P33" s="72"/>
+      <x:c r="O33" s="72" t="str"/>
+      <x:c r="P33" s="72" t="str"/>
       <x:c r="Q33" s="72" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2591,7 +2588,7 @@
       <x:c r="J34" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K34" s="76" t="n">
+      <x:c r="K34" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L34" s="76" t="str">
@@ -2603,8 +2600,8 @@
       <x:c r="N34" s="76" t="str">
         <x:v>https://stateparks.utah.gov/parks/jordanelle/</x:v>
       </x:c>
-      <x:c r="O34" s="76"/>
-      <x:c r="P34" s="76"/>
+      <x:c r="O34" s="76" t="str"/>
+      <x:c r="P34" s="76" t="str"/>
       <x:c r="Q34" s="76" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2640,7 +2637,7 @@
       <x:c r="J35" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="K35" s="72" t="n">
+      <x:c r="K35" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L35" s="72" t="str">
@@ -2649,7 +2646,7 @@
       <x:c r="M35" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N35" s="72"/>
+      <x:c r="N35" s="72" t="str"/>
       <x:c r="O35" s="72" t="str">
         <x:v>STREEX-owned original — Juan</x:v>
       </x:c>
@@ -2691,7 +2688,7 @@
       <x:c r="J36" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K36" s="76" t="n">
+      <x:c r="K36" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L36" s="76" t="str">
@@ -2703,8 +2700,8 @@
       <x:c r="N36" s="76" t="str">
         <x:v>https://www.egyptiantheatrecompany.org/</x:v>
       </x:c>
-      <x:c r="O36" s="76"/>
-      <x:c r="P36" s="76"/>
+      <x:c r="O36" s="76" t="str"/>
+      <x:c r="P36" s="76" t="str"/>
       <x:c r="Q36" s="76" t="str">
         <x:v>Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2731,14 +2728,14 @@
       <x:c r="G37" s="72" t="str">
         <x:v>utah-museum-of-fine-arts.jpg</x:v>
       </x:c>
-      <x:c r="H37" s="72"/>
+      <x:c r="H37" s="72" t="str"/>
       <x:c r="I37" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J37" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K37" s="72" t="n">
+      <x:c r="K37" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L37" s="72" t="str">
@@ -2750,8 +2747,8 @@
       <x:c r="N37" s="72" t="str">
         <x:v>https://www.umfa.utah.edu/</x:v>
       </x:c>
-      <x:c r="O37" s="72"/>
-      <x:c r="P37" s="72"/>
+      <x:c r="O37" s="72" t="str"/>
+      <x:c r="P37" s="72" t="str"/>
       <x:c r="Q37" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2778,14 +2775,14 @@
       <x:c r="G38" s="76" t="str">
         <x:v>the-leonardo.jpg</x:v>
       </x:c>
-      <x:c r="H38" s="76"/>
+      <x:c r="H38" s="76" t="str"/>
       <x:c r="I38" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J38" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K38" s="76" t="n">
+      <x:c r="K38" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L38" s="76" t="str">
@@ -2797,8 +2794,8 @@
       <x:c r="N38" s="76" t="str">
         <x:v>https://theleonardo.org/</x:v>
       </x:c>
-      <x:c r="O38" s="76"/>
-      <x:c r="P38" s="76"/>
+      <x:c r="O38" s="76" t="str"/>
+      <x:c r="P38" s="76" t="str"/>
       <x:c r="Q38" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2825,14 +2822,14 @@
       <x:c r="G39" s="72" t="str">
         <x:v>clark-planetarium.jpg</x:v>
       </x:c>
-      <x:c r="H39" s="72"/>
+      <x:c r="H39" s="72" t="str"/>
       <x:c r="I39" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J39" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K39" s="72" t="n">
+      <x:c r="K39" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L39" s="72" t="str">
@@ -2844,8 +2841,8 @@
       <x:c r="N39" s="72" t="str">
         <x:v>https://slplanet.com/</x:v>
       </x:c>
-      <x:c r="O39" s="72"/>
-      <x:c r="P39" s="72"/>
+      <x:c r="O39" s="72" t="str"/>
+      <x:c r="P39" s="72" t="str"/>
       <x:c r="Q39" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2872,14 +2869,14 @@
       <x:c r="G40" s="76" t="str">
         <x:v>discovery-gateway.jpg</x:v>
       </x:c>
-      <x:c r="H40" s="76"/>
+      <x:c r="H40" s="76" t="str"/>
       <x:c r="I40" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J40" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K40" s="76" t="n">
+      <x:c r="K40" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L40" s="76" t="str">
@@ -2891,8 +2888,8 @@
       <x:c r="N40" s="76" t="str">
         <x:v>https://discoverygateway.org/</x:v>
       </x:c>
-      <x:c r="O40" s="76"/>
-      <x:c r="P40" s="76"/>
+      <x:c r="O40" s="76" t="str"/>
+      <x:c r="P40" s="76" t="str"/>
       <x:c r="Q40" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2919,14 +2916,14 @@
       <x:c r="G41" s="72" t="str">
         <x:v>salt-palace-convention-center.jpg</x:v>
       </x:c>
-      <x:c r="H41" s="72"/>
+      <x:c r="H41" s="72" t="str"/>
       <x:c r="I41" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J41" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K41" s="72" t="n">
+      <x:c r="K41" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L41" s="72" t="str">
@@ -2938,8 +2935,8 @@
       <x:c r="N41" s="72" t="str">
         <x:v>https://www.visitsaltlake.com/</x:v>
       </x:c>
-      <x:c r="O41" s="72"/>
-      <x:c r="P41" s="72"/>
+      <x:c r="O41" s="72" t="str"/>
+      <x:c r="P41" s="72" t="str"/>
       <x:c r="Q41" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -2966,14 +2963,14 @@
       <x:c r="G42" s="76" t="str">
         <x:v>eccles-theater.jpg</x:v>
       </x:c>
-      <x:c r="H42" s="76"/>
+      <x:c r="H42" s="76" t="str"/>
       <x:c r="I42" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J42" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K42" s="76" t="n">
+      <x:c r="K42" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L42" s="76" t="str">
@@ -2985,8 +2982,8 @@
       <x:c r="N42" s="76" t="str">
         <x:v>https://www.eccles-theater.com/</x:v>
       </x:c>
-      <x:c r="O42" s="76"/>
-      <x:c r="P42" s="76"/>
+      <x:c r="O42" s="76" t="str"/>
+      <x:c r="P42" s="76" t="str"/>
       <x:c r="Q42" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3013,14 +3010,14 @@
       <x:c r="G43" s="72" t="str">
         <x:v>abravanel-hall.jpg</x:v>
       </x:c>
-      <x:c r="H43" s="72"/>
+      <x:c r="H43" s="72" t="str"/>
       <x:c r="I43" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J43" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K43" s="72" t="n">
+      <x:c r="K43" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L43" s="72" t="str">
@@ -3032,8 +3029,8 @@
       <x:c r="N43" s="72" t="str">
         <x:v>https://utaharts.org/</x:v>
       </x:c>
-      <x:c r="O43" s="72"/>
-      <x:c r="P43" s="72"/>
+      <x:c r="O43" s="72" t="str"/>
+      <x:c r="P43" s="72" t="str"/>
       <x:c r="Q43" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3060,14 +3057,14 @@
       <x:c r="G44" s="76" t="str">
         <x:v>delta-center.jpg</x:v>
       </x:c>
-      <x:c r="H44" s="76"/>
+      <x:c r="H44" s="76" t="str"/>
       <x:c r="I44" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J44" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K44" s="76" t="n">
+      <x:c r="K44" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L44" s="76" t="str">
@@ -3079,8 +3076,8 @@
       <x:c r="N44" s="76" t="str">
         <x:v>https://www.nba.com/jazz/arena</x:v>
       </x:c>
-      <x:c r="O44" s="76"/>
-      <x:c r="P44" s="76"/>
+      <x:c r="O44" s="76" t="str"/>
+      <x:c r="P44" s="76" t="str"/>
       <x:c r="Q44" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3107,14 +3104,14 @@
       <x:c r="G45" s="72" t="str">
         <x:v>rice-eccles-stadium.jpg</x:v>
       </x:c>
-      <x:c r="H45" s="72"/>
+      <x:c r="H45" s="72" t="str"/>
       <x:c r="I45" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J45" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K45" s="72" t="n">
+      <x:c r="K45" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L45" s="72" t="str">
@@ -3126,8 +3123,8 @@
       <x:c r="N45" s="72" t="str">
         <x:v>https://stadium.utah.edu/</x:v>
       </x:c>
-      <x:c r="O45" s="72"/>
-      <x:c r="P45" s="72"/>
+      <x:c r="O45" s="72" t="str"/>
+      <x:c r="P45" s="72" t="str"/>
       <x:c r="Q45" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3154,14 +3151,14 @@
       <x:c r="G46" s="76" t="str">
         <x:v>america-first-field.jpg</x:v>
       </x:c>
-      <x:c r="H46" s="76"/>
+      <x:c r="H46" s="76" t="str"/>
       <x:c r="I46" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J46" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K46" s="76" t="n">
+      <x:c r="K46" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L46" s="76" t="str">
@@ -3173,8 +3170,8 @@
       <x:c r="N46" s="76" t="str">
         <x:v>https://www.rsl.com/america-first-field</x:v>
       </x:c>
-      <x:c r="O46" s="76"/>
-      <x:c r="P46" s="76"/>
+      <x:c r="O46" s="76" t="str"/>
+      <x:c r="P46" s="76" t="str"/>
       <x:c r="Q46" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3201,14 +3198,14 @@
       <x:c r="G47" s="72" t="str">
         <x:v>maverik-stadium.jpg</x:v>
       </x:c>
-      <x:c r="H47" s="72"/>
+      <x:c r="H47" s="72" t="str"/>
       <x:c r="I47" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J47" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K47" s="72" t="n">
+      <x:c r="K47" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L47" s="72" t="str">
@@ -3220,8 +3217,8 @@
       <x:c r="N47" s="72" t="str">
         <x:v>https://utahstateaggies.com/facilities/maverik-stadium/</x:v>
       </x:c>
-      <x:c r="O47" s="72"/>
-      <x:c r="P47" s="72"/>
+      <x:c r="O47" s="72" t="str"/>
+      <x:c r="P47" s="72" t="str"/>
       <x:c r="Q47" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3248,14 +3245,14 @@
       <x:c r="G48" s="76" t="str">
         <x:v>utah-state-fairpark.jpg</x:v>
       </x:c>
-      <x:c r="H48" s="76"/>
+      <x:c r="H48" s="76" t="str"/>
       <x:c r="I48" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J48" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K48" s="76" t="n">
+      <x:c r="K48" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L48" s="76" t="str">
@@ -3267,8 +3264,8 @@
       <x:c r="N48" s="76" t="str">
         <x:v>https://utahstatefair.com/</x:v>
       </x:c>
-      <x:c r="O48" s="76"/>
-      <x:c r="P48" s="76"/>
+      <x:c r="O48" s="76" t="str"/>
+      <x:c r="P48" s="76" t="str"/>
       <x:c r="Q48" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3295,14 +3292,14 @@
       <x:c r="G49" s="72" t="str">
         <x:v>sugar-house-park.jpg</x:v>
       </x:c>
-      <x:c r="H49" s="72"/>
+      <x:c r="H49" s="72" t="str"/>
       <x:c r="I49" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J49" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K49" s="72" t="n">
+      <x:c r="K49" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L49" s="72" t="str">
@@ -3314,8 +3311,8 @@
       <x:c r="N49" s="72" t="str">
         <x:v>https://www.slc.gov/parks/</x:v>
       </x:c>
-      <x:c r="O49" s="72"/>
-      <x:c r="P49" s="72"/>
+      <x:c r="O49" s="72" t="str"/>
+      <x:c r="P49" s="72" t="str"/>
       <x:c r="Q49" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3342,14 +3339,14 @@
       <x:c r="G50" s="76" t="str">
         <x:v>9th-and-9th.jpg</x:v>
       </x:c>
-      <x:c r="H50" s="76"/>
+      <x:c r="H50" s="76" t="str"/>
       <x:c r="I50" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J50" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K50" s="76" t="n">
+      <x:c r="K50" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L50" s="76" t="str">
@@ -3361,8 +3358,8 @@
       <x:c r="N50" s="76" t="str">
         <x:v>https://www.visitsaltlake.com/</x:v>
       </x:c>
-      <x:c r="O50" s="76"/>
-      <x:c r="P50" s="76"/>
+      <x:c r="O50" s="76" t="str"/>
+      <x:c r="P50" s="76" t="str"/>
       <x:c r="Q50" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3389,14 +3386,14 @@
       <x:c r="G51" s="72" t="str">
         <x:v>the-avenues.jpg</x:v>
       </x:c>
-      <x:c r="H51" s="72"/>
+      <x:c r="H51" s="72" t="str"/>
       <x:c r="I51" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J51" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K51" s="72" t="n">
+      <x:c r="K51" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L51" s="72" t="str">
@@ -3408,8 +3405,8 @@
       <x:c r="N51" s="72" t="str">
         <x:v>https://www.slc.gov/</x:v>
       </x:c>
-      <x:c r="O51" s="72"/>
-      <x:c r="P51" s="72"/>
+      <x:c r="O51" s="72" t="str"/>
+      <x:c r="P51" s="72" t="str"/>
       <x:c r="Q51" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3436,14 +3433,14 @@
       <x:c r="G52" s="76" t="str">
         <x:v>memory-grove-park.jpg</x:v>
       </x:c>
-      <x:c r="H52" s="76"/>
+      <x:c r="H52" s="76" t="str"/>
       <x:c r="I52" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J52" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K52" s="76" t="n">
+      <x:c r="K52" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L52" s="76" t="str">
@@ -3455,8 +3452,8 @@
       <x:c r="N52" s="76" t="str">
         <x:v>https://www.slc.gov/parks/</x:v>
       </x:c>
-      <x:c r="O52" s="76"/>
-      <x:c r="P52" s="76"/>
+      <x:c r="O52" s="76" t="str"/>
+      <x:c r="P52" s="76" t="str"/>
       <x:c r="Q52" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3483,14 +3480,14 @@
       <x:c r="G53" s="72" t="str">
         <x:v>jordan-river-parkway.jpg</x:v>
       </x:c>
-      <x:c r="H53" s="72"/>
+      <x:c r="H53" s="72" t="str"/>
       <x:c r="I53" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J53" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K53" s="72" t="n">
+      <x:c r="K53" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L53" s="72" t="str">
@@ -3502,8 +3499,8 @@
       <x:c r="N53" s="72" t="str">
         <x:v>https://www.slc.gov/parks/</x:v>
       </x:c>
-      <x:c r="O53" s="72"/>
-      <x:c r="P53" s="72"/>
+      <x:c r="O53" s="72" t="str"/>
+      <x:c r="P53" s="72" t="str"/>
       <x:c r="Q53" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3530,14 +3527,14 @@
       <x:c r="G54" s="76" t="str">
         <x:v>bonneville-shoreline-trail.jpg</x:v>
       </x:c>
-      <x:c r="H54" s="76"/>
+      <x:c r="H54" s="76" t="str"/>
       <x:c r="I54" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J54" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K54" s="76" t="n">
+      <x:c r="K54" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L54" s="76" t="str">
@@ -3549,8 +3546,8 @@
       <x:c r="N54" s="76" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O54" s="76"/>
-      <x:c r="P54" s="76"/>
+      <x:c r="O54" s="76" t="str"/>
+      <x:c r="P54" s="76" t="str"/>
       <x:c r="Q54" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3577,14 +3574,14 @@
       <x:c r="G55" s="72" t="str">
         <x:v>big-cottonwood-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H55" s="72"/>
+      <x:c r="H55" s="72" t="str"/>
       <x:c r="I55" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J55" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K55" s="72" t="n">
+      <x:c r="K55" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L55" s="72" t="str">
@@ -3596,8 +3593,8 @@
       <x:c r="N55" s="72" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O55" s="72"/>
-      <x:c r="P55" s="72"/>
+      <x:c r="O55" s="72" t="str"/>
+      <x:c r="P55" s="72" t="str"/>
       <x:c r="Q55" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3624,14 +3621,14 @@
       <x:c r="G56" s="76" t="str">
         <x:v>little-cottonwood-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H56" s="76"/>
+      <x:c r="H56" s="76" t="str"/>
       <x:c r="I56" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J56" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K56" s="76" t="n">
+      <x:c r="K56" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L56" s="76" t="str">
@@ -3643,8 +3640,8 @@
       <x:c r="N56" s="76" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O56" s="76"/>
-      <x:c r="P56" s="76"/>
+      <x:c r="O56" s="76" t="str"/>
+      <x:c r="P56" s="76" t="str"/>
       <x:c r="Q56" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3671,14 +3668,14 @@
       <x:c r="G57" s="72" t="str">
         <x:v>millcreek-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H57" s="72"/>
+      <x:c r="H57" s="72" t="str"/>
       <x:c r="I57" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J57" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K57" s="72" t="n">
+      <x:c r="K57" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L57" s="72" t="str">
@@ -3690,8 +3687,8 @@
       <x:c r="N57" s="72" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O57" s="72"/>
-      <x:c r="P57" s="72"/>
+      <x:c r="O57" s="72" t="str"/>
+      <x:c r="P57" s="72" t="str"/>
       <x:c r="Q57" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3718,14 +3715,14 @@
       <x:c r="G58" s="76" t="str">
         <x:v>snowbird.jpg</x:v>
       </x:c>
-      <x:c r="H58" s="76"/>
+      <x:c r="H58" s="76" t="str"/>
       <x:c r="I58" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J58" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K58" s="76" t="n">
+      <x:c r="K58" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L58" s="76" t="str">
@@ -3737,8 +3734,8 @@
       <x:c r="N58" s="76" t="str">
         <x:v>https://www.snowbird.com/</x:v>
       </x:c>
-      <x:c r="O58" s="76"/>
-      <x:c r="P58" s="76"/>
+      <x:c r="O58" s="76" t="str"/>
+      <x:c r="P58" s="76" t="str"/>
       <x:c r="Q58" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3765,14 +3762,14 @@
       <x:c r="G59" s="72" t="str">
         <x:v>alta-ski-area.jpg</x:v>
       </x:c>
-      <x:c r="H59" s="72"/>
+      <x:c r="H59" s="72" t="str"/>
       <x:c r="I59" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J59" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K59" s="72" t="n">
+      <x:c r="K59" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L59" s="72" t="str">
@@ -3784,8 +3781,8 @@
       <x:c r="N59" s="72" t="str">
         <x:v>https://www.alta.com/</x:v>
       </x:c>
-      <x:c r="O59" s="72"/>
-      <x:c r="P59" s="72"/>
+      <x:c r="O59" s="72" t="str"/>
+      <x:c r="P59" s="72" t="str"/>
       <x:c r="Q59" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3812,14 +3809,14 @@
       <x:c r="G60" s="76" t="str">
         <x:v>solitude-mountain-resort.jpg</x:v>
       </x:c>
-      <x:c r="H60" s="76"/>
+      <x:c r="H60" s="76" t="str"/>
       <x:c r="I60" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J60" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K60" s="76" t="n">
+      <x:c r="K60" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L60" s="76" t="str">
@@ -3831,8 +3828,8 @@
       <x:c r="N60" s="76" t="str">
         <x:v>https://www.solitudemountain.com/</x:v>
       </x:c>
-      <x:c r="O60" s="76"/>
-      <x:c r="P60" s="76"/>
+      <x:c r="O60" s="76" t="str"/>
+      <x:c r="P60" s="76" t="str"/>
       <x:c r="Q60" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3859,14 +3856,14 @@
       <x:c r="G61" s="72" t="str">
         <x:v>brighton-resort.jpg</x:v>
       </x:c>
-      <x:c r="H61" s="72"/>
+      <x:c r="H61" s="72" t="str"/>
       <x:c r="I61" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J61" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K61" s="72" t="n">
+      <x:c r="K61" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L61" s="72" t="str">
@@ -3878,8 +3875,8 @@
       <x:c r="N61" s="72" t="str">
         <x:v>https://brightonresort.com/</x:v>
       </x:c>
-      <x:c r="O61" s="72"/>
-      <x:c r="P61" s="72"/>
+      <x:c r="O61" s="72" t="str"/>
+      <x:c r="P61" s="72" t="str"/>
       <x:c r="Q61" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3906,14 +3903,14 @@
       <x:c r="G62" s="76" t="str">
         <x:v>snowbasin-resort.jpg</x:v>
       </x:c>
-      <x:c r="H62" s="76"/>
+      <x:c r="H62" s="76" t="str"/>
       <x:c r="I62" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J62" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K62" s="76" t="n">
+      <x:c r="K62" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L62" s="76" t="str">
@@ -3925,8 +3922,8 @@
       <x:c r="N62" s="76" t="str">
         <x:v>https://www.snowbasin.com/</x:v>
       </x:c>
-      <x:c r="O62" s="76"/>
-      <x:c r="P62" s="76"/>
+      <x:c r="O62" s="76" t="str"/>
+      <x:c r="P62" s="76" t="str"/>
       <x:c r="Q62" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -3953,14 +3950,14 @@
       <x:c r="G63" s="72" t="str">
         <x:v>powder-mountain.jpg</x:v>
       </x:c>
-      <x:c r="H63" s="72"/>
+      <x:c r="H63" s="72" t="str"/>
       <x:c r="I63" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J63" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K63" s="72" t="n">
+      <x:c r="K63" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L63" s="72" t="str">
@@ -3972,8 +3969,8 @@
       <x:c r="N63" s="72" t="str">
         <x:v>https://www.powdermountain.com/</x:v>
       </x:c>
-      <x:c r="O63" s="72"/>
-      <x:c r="P63" s="72"/>
+      <x:c r="O63" s="72" t="str"/>
+      <x:c r="P63" s="72" t="str"/>
       <x:c r="Q63" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4000,14 +3997,14 @@
       <x:c r="G64" s="76" t="str">
         <x:v>canyons-village.jpg</x:v>
       </x:c>
-      <x:c r="H64" s="76"/>
+      <x:c r="H64" s="76" t="str"/>
       <x:c r="I64" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J64" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K64" s="76" t="n">
+      <x:c r="K64" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L64" s="76" t="str">
@@ -4019,8 +4016,8 @@
       <x:c r="N64" s="76" t="str">
         <x:v>https://www.visitparkcity.com/</x:v>
       </x:c>
-      <x:c r="O64" s="76"/>
-      <x:c r="P64" s="76"/>
+      <x:c r="O64" s="76" t="str"/>
+      <x:c r="P64" s="76" t="str"/>
       <x:c r="Q64" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4047,14 +4044,14 @@
       <x:c r="G65" s="72" t="str">
         <x:v>park-city-mountain.jpg</x:v>
       </x:c>
-      <x:c r="H65" s="72"/>
+      <x:c r="H65" s="72" t="str"/>
       <x:c r="I65" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J65" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K65" s="72" t="n">
+      <x:c r="K65" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L65" s="72" t="str">
@@ -4066,8 +4063,8 @@
       <x:c r="N65" s="72" t="str">
         <x:v>https://www.visitparkcity.com/</x:v>
       </x:c>
-      <x:c r="O65" s="72"/>
-      <x:c r="P65" s="72"/>
+      <x:c r="O65" s="72" t="str"/>
+      <x:c r="P65" s="72" t="str"/>
       <x:c r="Q65" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4094,14 +4091,14 @@
       <x:c r="G66" s="76" t="str">
         <x:v>park-city-library.jpg</x:v>
       </x:c>
-      <x:c r="H66" s="76"/>
+      <x:c r="H66" s="76" t="str"/>
       <x:c r="I66" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J66" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K66" s="76" t="n">
+      <x:c r="K66" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L66" s="76" t="str">
@@ -4113,8 +4110,8 @@
       <x:c r="N66" s="76" t="str">
         <x:v>https://www.visitparkcity.com/</x:v>
       </x:c>
-      <x:c r="O66" s="76"/>
-      <x:c r="P66" s="76"/>
+      <x:c r="O66" s="76" t="str"/>
+      <x:c r="P66" s="76" t="str"/>
       <x:c r="Q66" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4141,14 +4138,14 @@
       <x:c r="G67" s="72" t="str">
         <x:v>park-city-museum.jpg</x:v>
       </x:c>
-      <x:c r="H67" s="72"/>
+      <x:c r="H67" s="72" t="str"/>
       <x:c r="I67" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J67" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K67" s="72" t="n">
+      <x:c r="K67" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L67" s="72" t="str">
@@ -4160,8 +4157,8 @@
       <x:c r="N67" s="72" t="str">
         <x:v>https://www.parkcityhistory.org/</x:v>
       </x:c>
-      <x:c r="O67" s="72"/>
-      <x:c r="P67" s="72"/>
+      <x:c r="O67" s="72" t="str"/>
+      <x:c r="P67" s="72" t="str"/>
       <x:c r="Q67" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4188,14 +4185,14 @@
       <x:c r="G68" s="76" t="str">
         <x:v>woodward-park-city.jpg</x:v>
       </x:c>
-      <x:c r="H68" s="76"/>
+      <x:c r="H68" s="76" t="str"/>
       <x:c r="I68" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J68" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K68" s="76" t="n">
+      <x:c r="K68" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L68" s="76" t="str">
@@ -4207,8 +4204,8 @@
       <x:c r="N68" s="76" t="str">
         <x:v>https://woodwardparkcity.com/</x:v>
       </x:c>
-      <x:c r="O68" s="76"/>
-      <x:c r="P68" s="76"/>
+      <x:c r="O68" s="76" t="str"/>
+      <x:c r="P68" s="76" t="str"/>
       <x:c r="Q68" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4235,14 +4232,14 @@
       <x:c r="G69" s="72" t="str">
         <x:v>heber-valley-railroad.jpg</x:v>
       </x:c>
-      <x:c r="H69" s="72"/>
+      <x:c r="H69" s="72" t="str"/>
       <x:c r="I69" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J69" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K69" s="72" t="n">
+      <x:c r="K69" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L69" s="72" t="str">
@@ -4254,8 +4251,8 @@
       <x:c r="N69" s="72" t="str">
         <x:v>https://www.hebervalleyrr.org/</x:v>
       </x:c>
-      <x:c r="O69" s="72"/>
-      <x:c r="P69" s="72"/>
+      <x:c r="O69" s="72" t="str"/>
+      <x:c r="P69" s="72" t="str"/>
       <x:c r="Q69" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4282,14 +4279,14 @@
       <x:c r="G70" s="76" t="str">
         <x:v>deer-creek-reservoir.jpg</x:v>
       </x:c>
-      <x:c r="H70" s="76"/>
+      <x:c r="H70" s="76" t="str"/>
       <x:c r="I70" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J70" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K70" s="76" t="n">
+      <x:c r="K70" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L70" s="76" t="str">
@@ -4301,8 +4298,8 @@
       <x:c r="N70" s="76" t="str">
         <x:v>https://stateparks.utah.gov/</x:v>
       </x:c>
-      <x:c r="O70" s="76"/>
-      <x:c r="P70" s="76"/>
+      <x:c r="O70" s="76" t="str"/>
+      <x:c r="P70" s="76" t="str"/>
       <x:c r="Q70" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4329,14 +4326,14 @@
       <x:c r="G71" s="72" t="str">
         <x:v>provo-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H71" s="72"/>
+      <x:c r="H71" s="72" t="str"/>
       <x:c r="I71" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J71" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K71" s="72" t="n">
+      <x:c r="K71" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L71" s="72" t="str">
@@ -4348,8 +4345,8 @@
       <x:c r="N71" s="72" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O71" s="72"/>
-      <x:c r="P71" s="72"/>
+      <x:c r="O71" s="72" t="str"/>
+      <x:c r="P71" s="72" t="str"/>
       <x:c r="Q71" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4376,14 +4373,14 @@
       <x:c r="G72" s="76" t="str">
         <x:v>bridal-veil-falls.jpg</x:v>
       </x:c>
-      <x:c r="H72" s="76"/>
+      <x:c r="H72" s="76" t="str"/>
       <x:c r="I72" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J72" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K72" s="76" t="n">
+      <x:c r="K72" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L72" s="76" t="str">
@@ -4395,8 +4392,8 @@
       <x:c r="N72" s="76" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O72" s="76"/>
-      <x:c r="P72" s="76"/>
+      <x:c r="O72" s="76" t="str"/>
+      <x:c r="P72" s="76" t="str"/>
       <x:c r="Q72" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4423,14 +4420,14 @@
       <x:c r="G73" s="72" t="str">
         <x:v>mount-timpanogos.jpg</x:v>
       </x:c>
-      <x:c r="H73" s="72"/>
+      <x:c r="H73" s="72" t="str"/>
       <x:c r="I73" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J73" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K73" s="72" t="n">
+      <x:c r="K73" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L73" s="72" t="str">
@@ -4442,8 +4439,8 @@
       <x:c r="N73" s="72" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O73" s="72"/>
-      <x:c r="P73" s="72"/>
+      <x:c r="O73" s="72" t="str"/>
+      <x:c r="P73" s="72" t="str"/>
       <x:c r="Q73" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4470,14 +4467,14 @@
       <x:c r="G74" s="76" t="str">
         <x:v>ogden-union-station.jpg</x:v>
       </x:c>
-      <x:c r="H74" s="76"/>
+      <x:c r="H74" s="76" t="str"/>
       <x:c r="I74" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J74" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K74" s="76" t="n">
+      <x:c r="K74" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L74" s="76" t="str">
@@ -4489,8 +4486,8 @@
       <x:c r="N74" s="76" t="str">
         <x:v>https://www.visitogden.com/</x:v>
       </x:c>
-      <x:c r="O74" s="76"/>
-      <x:c r="P74" s="76"/>
+      <x:c r="O74" s="76" t="str"/>
+      <x:c r="P74" s="76" t="str"/>
       <x:c r="Q74" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4517,14 +4514,14 @@
       <x:c r="G75" s="72" t="str">
         <x:v>eccles-dinosaur-park.jpg</x:v>
       </x:c>
-      <x:c r="H75" s="72"/>
+      <x:c r="H75" s="72" t="str"/>
       <x:c r="I75" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J75" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K75" s="72" t="n">
+      <x:c r="K75" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L75" s="72" t="str">
@@ -4536,8 +4533,8 @@
       <x:c r="N75" s="72" t="str">
         <x:v>https://dinosaurpark.org/</x:v>
       </x:c>
-      <x:c r="O75" s="72"/>
-      <x:c r="P75" s="72"/>
+      <x:c r="O75" s="72" t="str"/>
+      <x:c r="P75" s="72" t="str"/>
       <x:c r="Q75" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4564,14 +4561,14 @@
       <x:c r="G76" s="76" t="str">
         <x:v>ogden-nature-center.jpg</x:v>
       </x:c>
-      <x:c r="H76" s="76"/>
+      <x:c r="H76" s="76" t="str"/>
       <x:c r="I76" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J76" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K76" s="76" t="n">
+      <x:c r="K76" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L76" s="76" t="str">
@@ -4583,8 +4580,8 @@
       <x:c r="N76" s="76" t="str">
         <x:v>https://ogdennaturecenter.org/</x:v>
       </x:c>
-      <x:c r="O76" s="76"/>
-      <x:c r="P76" s="76"/>
+      <x:c r="O76" s="76" t="str"/>
+      <x:c r="P76" s="76" t="str"/>
       <x:c r="Q76" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4611,14 +4608,14 @@
       <x:c r="G77" s="72" t="str">
         <x:v>25th-street-historic-district.jpg</x:v>
       </x:c>
-      <x:c r="H77" s="72"/>
+      <x:c r="H77" s="72" t="str"/>
       <x:c r="I77" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J77" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K77" s="72" t="n">
+      <x:c r="K77" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L77" s="72" t="str">
@@ -4630,8 +4627,8 @@
       <x:c r="N77" s="72" t="str">
         <x:v>https://www.visitogden.com/</x:v>
       </x:c>
-      <x:c r="O77" s="72"/>
-      <x:c r="P77" s="72"/>
+      <x:c r="O77" s="72" t="str"/>
+      <x:c r="P77" s="72" t="str"/>
       <x:c r="Q77" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4658,14 +4655,14 @@
       <x:c r="G78" s="76" t="str">
         <x:v>hill-aerospace-museum.jpg</x:v>
       </x:c>
-      <x:c r="H78" s="76"/>
+      <x:c r="H78" s="76" t="str"/>
       <x:c r="I78" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J78" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K78" s="76" t="n">
+      <x:c r="K78" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L78" s="76" t="str">
@@ -4677,8 +4674,8 @@
       <x:c r="N78" s="76" t="str">
         <x:v>https://www.aerospaceutah.com/</x:v>
       </x:c>
-      <x:c r="O78" s="76"/>
-      <x:c r="P78" s="76"/>
+      <x:c r="O78" s="76" t="str"/>
+      <x:c r="P78" s="76" t="str"/>
       <x:c r="Q78" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4705,14 +4702,14 @@
       <x:c r="G79" s="72" t="str">
         <x:v>salomon-center.jpg</x:v>
       </x:c>
-      <x:c r="H79" s="72"/>
+      <x:c r="H79" s="72" t="str"/>
       <x:c r="I79" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J79" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K79" s="72" t="n">
+      <x:c r="K79" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L79" s="72" t="str">
@@ -4724,8 +4721,8 @@
       <x:c r="N79" s="72" t="str">
         <x:v>https://www.visitogden.com/</x:v>
       </x:c>
-      <x:c r="O79" s="72"/>
-      <x:c r="P79" s="72"/>
+      <x:c r="O79" s="72" t="str"/>
+      <x:c r="P79" s="72" t="str"/>
       <x:c r="Q79" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4752,14 +4749,14 @@
       <x:c r="G80" s="76" t="str">
         <x:v>weber-state-university.jpg</x:v>
       </x:c>
-      <x:c r="H80" s="76"/>
+      <x:c r="H80" s="76" t="str"/>
       <x:c r="I80" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J80" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K80" s="76" t="n">
+      <x:c r="K80" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L80" s="76" t="str">
@@ -4771,8 +4768,8 @@
       <x:c r="N80" s="76" t="str">
         <x:v>https://www.weber.edu/</x:v>
       </x:c>
-      <x:c r="O80" s="76"/>
-      <x:c r="P80" s="76"/>
+      <x:c r="O80" s="76" t="str"/>
+      <x:c r="P80" s="76" t="str"/>
       <x:c r="Q80" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4799,14 +4796,14 @@
       <x:c r="G81" s="72" t="str">
         <x:v>ogden-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H81" s="72"/>
+      <x:c r="H81" s="72" t="str"/>
       <x:c r="I81" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J81" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K81" s="72" t="n">
+      <x:c r="K81" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L81" s="72" t="str">
@@ -4818,8 +4815,8 @@
       <x:c r="N81" s="72" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O81" s="72"/>
-      <x:c r="P81" s="72"/>
+      <x:c r="O81" s="72" t="str"/>
+      <x:c r="P81" s="72" t="str"/>
       <x:c r="Q81" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4846,14 +4843,14 @@
       <x:c r="G82" s="76" t="str">
         <x:v>pineview-reservoir.jpg</x:v>
       </x:c>
-      <x:c r="H82" s="76"/>
+      <x:c r="H82" s="76" t="str"/>
       <x:c r="I82" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J82" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K82" s="76" t="n">
+      <x:c r="K82" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L82" s="76" t="str">
@@ -4865,8 +4862,8 @@
       <x:c r="N82" s="76" t="str">
         <x:v>https://www.visitogden.com/</x:v>
       </x:c>
-      <x:c r="O82" s="76"/>
-      <x:c r="P82" s="76"/>
+      <x:c r="O82" s="76" t="str"/>
+      <x:c r="P82" s="76" t="str"/>
       <x:c r="Q82" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4893,14 +4890,14 @@
       <x:c r="G83" s="72" t="str">
         <x:v>fielding-garr-ranch.jpg</x:v>
       </x:c>
-      <x:c r="H83" s="72"/>
+      <x:c r="H83" s="72" t="str"/>
       <x:c r="I83" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J83" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K83" s="72" t="n">
+      <x:c r="K83" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L83" s="72" t="str">
@@ -4912,8 +4909,8 @@
       <x:c r="N83" s="72" t="str">
         <x:v>https://stateparks.utah.gov/parks/antelope-island/</x:v>
       </x:c>
-      <x:c r="O83" s="72"/>
-      <x:c r="P83" s="72"/>
+      <x:c r="O83" s="72" t="str"/>
+      <x:c r="P83" s="72" t="str"/>
       <x:c r="Q83" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4940,14 +4937,14 @@
       <x:c r="G84" s="76" t="str">
         <x:v>saltair.jpg</x:v>
       </x:c>
-      <x:c r="H84" s="76"/>
+      <x:c r="H84" s="76" t="str"/>
       <x:c r="I84" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J84" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K84" s="76" t="n">
+      <x:c r="K84" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L84" s="76" t="str">
@@ -4959,8 +4956,8 @@
       <x:c r="N84" s="76" t="str">
         <x:v>https://saltairutah.com/</x:v>
       </x:c>
-      <x:c r="O84" s="76"/>
-      <x:c r="P84" s="76"/>
+      <x:c r="O84" s="76" t="str"/>
+      <x:c r="P84" s="76" t="str"/>
       <x:c r="Q84" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -4987,14 +4984,14 @@
       <x:c r="G85" s="72" t="str">
         <x:v>spiral-jetty.jpg</x:v>
       </x:c>
-      <x:c r="H85" s="72"/>
+      <x:c r="H85" s="72" t="str"/>
       <x:c r="I85" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J85" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K85" s="72" t="n">
+      <x:c r="K85" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L85" s="72" t="str">
@@ -5006,8 +5003,8 @@
       <x:c r="N85" s="72" t="str">
         <x:v>https://www.utah.com/</x:v>
       </x:c>
-      <x:c r="O85" s="72"/>
-      <x:c r="P85" s="72"/>
+      <x:c r="O85" s="72" t="str"/>
+      <x:c r="P85" s="72" t="str"/>
       <x:c r="Q85" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5034,14 +5031,14 @@
       <x:c r="G86" s="76" t="str">
         <x:v>bonneville-salt-flats.jpg</x:v>
       </x:c>
-      <x:c r="H86" s="76"/>
+      <x:c r="H86" s="76" t="str"/>
       <x:c r="I86" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J86" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K86" s="76" t="n">
+      <x:c r="K86" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L86" s="76" t="str">
@@ -5053,8 +5050,8 @@
       <x:c r="N86" s="76" t="str">
         <x:v>https://stateparks.utah.gov/</x:v>
       </x:c>
-      <x:c r="O86" s="76"/>
-      <x:c r="P86" s="76"/>
+      <x:c r="O86" s="76" t="str"/>
+      <x:c r="P86" s="76" t="str"/>
       <x:c r="Q86" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5081,14 +5078,14 @@
       <x:c r="G87" s="72" t="str">
         <x:v>farmington-bay.jpg</x:v>
       </x:c>
-      <x:c r="H87" s="72"/>
+      <x:c r="H87" s="72" t="str"/>
       <x:c r="I87" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J87" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K87" s="72" t="n">
+      <x:c r="K87" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L87" s="72" t="str">
@@ -5100,8 +5097,8 @@
       <x:c r="N87" s="72" t="str">
         <x:v>https://www.visitutah.com/</x:v>
       </x:c>
-      <x:c r="O87" s="72"/>
-      <x:c r="P87" s="72"/>
+      <x:c r="O87" s="72" t="str"/>
+      <x:c r="P87" s="72" t="str"/>
       <x:c r="Q87" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5128,14 +5125,14 @@
       <x:c r="G88" s="76" t="str">
         <x:v>bountiful.jpg</x:v>
       </x:c>
-      <x:c r="H88" s="76"/>
+      <x:c r="H88" s="76" t="str"/>
       <x:c r="I88" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J88" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K88" s="76" t="n">
+      <x:c r="K88" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L88" s="76" t="str">
@@ -5147,8 +5144,8 @@
       <x:c r="N88" s="76" t="str">
         <x:v>https://www.visitutah.com/</x:v>
       </x:c>
-      <x:c r="O88" s="76"/>
-      <x:c r="P88" s="76"/>
+      <x:c r="O88" s="76" t="str"/>
+      <x:c r="P88" s="76" t="str"/>
       <x:c r="Q88" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5175,14 +5172,14 @@
       <x:c r="G89" s="72" t="str">
         <x:v>kaysville.jpg</x:v>
       </x:c>
-      <x:c r="H89" s="72"/>
+      <x:c r="H89" s="72" t="str"/>
       <x:c r="I89" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J89" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K89" s="72" t="n">
+      <x:c r="K89" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L89" s="72" t="str">
@@ -5194,8 +5191,8 @@
       <x:c r="N89" s="72" t="str">
         <x:v>https://www.visitutah.com/</x:v>
       </x:c>
-      <x:c r="O89" s="72"/>
-      <x:c r="P89" s="72"/>
+      <x:c r="O89" s="72" t="str"/>
+      <x:c r="P89" s="72" t="str"/>
       <x:c r="Q89" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5222,14 +5219,14 @@
       <x:c r="G90" s="76" t="str">
         <x:v>layton.jpg</x:v>
       </x:c>
-      <x:c r="H90" s="76"/>
+      <x:c r="H90" s="76" t="str"/>
       <x:c r="I90" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J90" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K90" s="76" t="n">
+      <x:c r="K90" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L90" s="76" t="str">
@@ -5241,8 +5238,8 @@
       <x:c r="N90" s="76" t="str">
         <x:v>https://www.visitutah.com/</x:v>
       </x:c>
-      <x:c r="O90" s="76"/>
-      <x:c r="P90" s="76"/>
+      <x:c r="O90" s="76" t="str"/>
+      <x:c r="P90" s="76" t="str"/>
       <x:c r="Q90" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5269,14 +5266,14 @@
       <x:c r="G91" s="72" t="str">
         <x:v>station-park-farmington.jpg</x:v>
       </x:c>
-      <x:c r="H91" s="72"/>
+      <x:c r="H91" s="72" t="str"/>
       <x:c r="I91" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J91" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K91" s="72" t="n">
+      <x:c r="K91" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L91" s="72" t="str">
@@ -5288,8 +5285,8 @@
       <x:c r="N91" s="72" t="str">
         <x:v>https://www.stationpark.com/</x:v>
       </x:c>
-      <x:c r="O91" s="72"/>
-      <x:c r="P91" s="72"/>
+      <x:c r="O91" s="72" t="str"/>
+      <x:c r="P91" s="72" t="str"/>
       <x:c r="Q91" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5316,14 +5313,14 @@
       <x:c r="G92" s="76" t="str">
         <x:v>city-creek-center.jpg</x:v>
       </x:c>
-      <x:c r="H92" s="76"/>
+      <x:c r="H92" s="76" t="str"/>
       <x:c r="I92" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J92" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K92" s="76" t="n">
+      <x:c r="K92" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L92" s="76" t="str">
@@ -5335,8 +5332,8 @@
       <x:c r="N92" s="76" t="str">
         <x:v>https://www.shopcitycreekcenter.com/</x:v>
       </x:c>
-      <x:c r="O92" s="76"/>
-      <x:c r="P92" s="76"/>
+      <x:c r="O92" s="76" t="str"/>
+      <x:c r="P92" s="76" t="str"/>
       <x:c r="Q92" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5363,14 +5360,14 @@
       <x:c r="G93" s="72" t="str">
         <x:v>trolley-square.jpg</x:v>
       </x:c>
-      <x:c r="H93" s="72"/>
+      <x:c r="H93" s="72" t="str"/>
       <x:c r="I93" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J93" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K93" s="72" t="n">
+      <x:c r="K93" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L93" s="72" t="str">
@@ -5382,8 +5379,8 @@
       <x:c r="N93" s="72" t="str">
         <x:v>https://www.trolleysquare.com/</x:v>
       </x:c>
-      <x:c r="O93" s="72"/>
-      <x:c r="P93" s="72"/>
+      <x:c r="O93" s="72" t="str"/>
+      <x:c r="P93" s="72" t="str"/>
       <x:c r="Q93" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5410,14 +5407,14 @@
       <x:c r="G94" s="76" t="str">
         <x:v>900-south-historic-district.jpg</x:v>
       </x:c>
-      <x:c r="H94" s="76"/>
+      <x:c r="H94" s="76" t="str"/>
       <x:c r="I94" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J94" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K94" s="76" t="n">
+      <x:c r="K94" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L94" s="76" t="str">
@@ -5429,8 +5426,8 @@
       <x:c r="N94" s="76" t="str">
         <x:v>https://www.slc.gov/</x:v>
       </x:c>
-      <x:c r="O94" s="76"/>
-      <x:c r="P94" s="76"/>
+      <x:c r="O94" s="76" t="str"/>
+      <x:c r="P94" s="76" t="str"/>
       <x:c r="Q94" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5457,14 +5454,14 @@
       <x:c r="G95" s="72" t="str">
         <x:v>sugar-house.jpg</x:v>
       </x:c>
-      <x:c r="H95" s="72"/>
+      <x:c r="H95" s="72" t="str"/>
       <x:c r="I95" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J95" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K95" s="72" t="n">
+      <x:c r="K95" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L95" s="72" t="str">
@@ -5476,8 +5473,8 @@
       <x:c r="N95" s="72" t="str">
         <x:v>https://www.slc.gov/</x:v>
       </x:c>
-      <x:c r="O95" s="72"/>
-      <x:c r="P95" s="72"/>
+      <x:c r="O95" s="72" t="str"/>
+      <x:c r="P95" s="72" t="str"/>
       <x:c r="Q95" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5504,14 +5501,14 @@
       <x:c r="G96" s="76" t="str">
         <x:v>holladay.jpg</x:v>
       </x:c>
-      <x:c r="H96" s="76"/>
+      <x:c r="H96" s="76" t="str"/>
       <x:c r="I96" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J96" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K96" s="76" t="n">
+      <x:c r="K96" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L96" s="76" t="str">
@@ -5523,8 +5520,8 @@
       <x:c r="N96" s="76" t="str">
         <x:v>https://www.holladayut.gov/</x:v>
       </x:c>
-      <x:c r="O96" s="76"/>
-      <x:c r="P96" s="76"/>
+      <x:c r="O96" s="76" t="str"/>
+      <x:c r="P96" s="76" t="str"/>
       <x:c r="Q96" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5551,14 +5548,14 @@
       <x:c r="G97" s="72" t="str">
         <x:v>draper.jpg</x:v>
       </x:c>
-      <x:c r="H97" s="72"/>
+      <x:c r="H97" s="72" t="str"/>
       <x:c r="I97" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J97" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K97" s="72" t="n">
+      <x:c r="K97" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L97" s="72" t="str">
@@ -5570,8 +5567,8 @@
       <x:c r="N97" s="72" t="str">
         <x:v>https://www.draperutah.gov/</x:v>
       </x:c>
-      <x:c r="O97" s="72"/>
-      <x:c r="P97" s="72"/>
+      <x:c r="O97" s="72" t="str"/>
+      <x:c r="P97" s="72" t="str"/>
       <x:c r="Q97" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5598,14 +5595,14 @@
       <x:c r="G98" s="76" t="str">
         <x:v>sandy.jpg</x:v>
       </x:c>
-      <x:c r="H98" s="76"/>
+      <x:c r="H98" s="76" t="str"/>
       <x:c r="I98" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J98" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K98" s="76" t="n">
+      <x:c r="K98" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L98" s="76" t="str">
@@ -5617,8 +5614,8 @@
       <x:c r="N98" s="76" t="str">
         <x:v>https://www.sandy.utah.gov/</x:v>
       </x:c>
-      <x:c r="O98" s="76"/>
-      <x:c r="P98" s="76"/>
+      <x:c r="O98" s="76" t="str"/>
+      <x:c r="P98" s="76" t="str"/>
       <x:c r="Q98" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5645,14 +5642,14 @@
       <x:c r="G99" s="72" t="str">
         <x:v>mountain-dell-reservoir.jpg</x:v>
       </x:c>
-      <x:c r="H99" s="72"/>
+      <x:c r="H99" s="72" t="str"/>
       <x:c r="I99" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J99" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K99" s="72" t="n">
+      <x:c r="K99" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L99" s="72" t="str">
@@ -5664,8 +5661,8 @@
       <x:c r="N99" s="72" t="str">
         <x:v>https://www.slc.gov/parks/</x:v>
       </x:c>
-      <x:c r="O99" s="72"/>
-      <x:c r="P99" s="72"/>
+      <x:c r="O99" s="72" t="str"/>
+      <x:c r="P99" s="72" t="str"/>
       <x:c r="Q99" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5692,14 +5689,14 @@
       <x:c r="G100" s="76" t="str">
         <x:v>emigration-canyon.jpg</x:v>
       </x:c>
-      <x:c r="H100" s="76"/>
+      <x:c r="H100" s="76" t="str"/>
       <x:c r="I100" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J100" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K100" s="76" t="n">
+      <x:c r="K100" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L100" s="76" t="str">
@@ -5711,8 +5708,8 @@
       <x:c r="N100" s="76" t="str">
         <x:v>https://www.fs.usda.gov/</x:v>
       </x:c>
-      <x:c r="O100" s="76"/>
-      <x:c r="P100" s="76"/>
+      <x:c r="O100" s="76" t="str"/>
+      <x:c r="P100" s="76" t="str"/>
       <x:c r="Q100" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5739,14 +5736,14 @@
       <x:c r="G101" s="72" t="str">
         <x:v>thanksgiving-point.jpg</x:v>
       </x:c>
-      <x:c r="H101" s="72"/>
+      <x:c r="H101" s="72" t="str"/>
       <x:c r="I101" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J101" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K101" s="72" t="n">
+      <x:c r="K101" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L101" s="72" t="str">
@@ -5758,8 +5755,8 @@
       <x:c r="N101" s="72" t="str">
         <x:v>https://www.thanksgivingpoint.org/</x:v>
       </x:c>
-      <x:c r="O101" s="72"/>
-      <x:c r="P101" s="72"/>
+      <x:c r="O101" s="72" t="str"/>
+      <x:c r="P101" s="72" t="str"/>
       <x:c r="Q101" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5786,14 +5783,14 @@
       <x:c r="G102" s="76" t="str">
         <x:v>loveland-living-planet-aquarium.jpg</x:v>
       </x:c>
-      <x:c r="H102" s="76"/>
+      <x:c r="H102" s="76" t="str"/>
       <x:c r="I102" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J102" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K102" s="76" t="n">
+      <x:c r="K102" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L102" s="76" t="str">
@@ -5805,8 +5802,8 @@
       <x:c r="N102" s="76" t="str">
         <x:v>https://livingplanetaquarium.org/</x:v>
       </x:c>
-      <x:c r="O102" s="76"/>
-      <x:c r="P102" s="76"/>
+      <x:c r="O102" s="76" t="str"/>
+      <x:c r="P102" s="76" t="str"/>
       <x:c r="Q102" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5833,14 +5830,14 @@
       <x:c r="G103" s="72" t="str">
         <x:v>provo.jpg</x:v>
       </x:c>
-      <x:c r="H103" s="72"/>
+      <x:c r="H103" s="72" t="str"/>
       <x:c r="I103" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J103" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K103" s="72" t="n">
+      <x:c r="K103" s="72" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L103" s="72" t="str">
@@ -5852,8 +5849,8 @@
       <x:c r="N103" s="72" t="str">
         <x:v>https://www.provo.org/</x:v>
       </x:c>
-      <x:c r="O103" s="72"/>
-      <x:c r="P103" s="72"/>
+      <x:c r="O103" s="72" t="str"/>
+      <x:c r="P103" s="72" t="str"/>
       <x:c r="Q103" s="72" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>
@@ -5880,14 +5877,14 @@
       <x:c r="G104" s="76" t="str">
         <x:v>brigham-young-university.jpg</x:v>
       </x:c>
-      <x:c r="H104" s="76"/>
+      <x:c r="H104" s="76" t="str"/>
       <x:c r="I104" s="81" t="str">
         <x:v>Missing original</x:v>
       </x:c>
       <x:c r="J104" s="79" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="K104" s="76" t="n">
+      <x:c r="K104" s="76" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L104" s="76" t="str">
@@ -5899,8 +5896,8 @@
       <x:c r="N104" s="76" t="str">
         <x:v>https://www.byu.edu/</x:v>
       </x:c>
-      <x:c r="O104" s="76"/>
-      <x:c r="P104" s="76"/>
+      <x:c r="O104" s="76" t="str"/>
+      <x:c r="P104" s="76" t="str"/>
       <x:c r="Q104" s="76" t="str">
         <x:v>Candidate for later local catalog import; confirm GPS trigger radius and image rights before enabling. Keep one landscape hero image; aim for a 16:9-ish crop, landmark clearly visible, no text overlays or identifiable people as the main subject.</x:v>
       </x:c>

</xml_diff>

<commit_message>
Correct Around You image attribution and inventory
</commit_message>
<xml_diff>
--- a/assets-source/passenger/around-you/around-you-image-inventory.xlsx
+++ b/assets-source/passenger/around-you/around-you-image-inventory.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4a7060fa3f29475e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="R3e0fa0629b684141"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6f07752f17554c34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="R6dc2f67901b245d8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1103,13 +1103,13 @@
         <x:v>salt-lake-valley.jpg</x:v>
       </x:c>
       <x:c r="H5" s="72" t="str">
-        <x:v>/images/passenger/around-you/user/salt-lake-valley-juan.webp</x:v>
+        <x:v>/images/passenger/around-you/salt-lake-valley.webp</x:v>
       </x:c>
       <x:c r="I5" s="74" t="str">
-        <x:v>Own local asset</x:v>
+        <x:v>Shared fallback</x:v>
       </x:c>
       <x:c r="J5" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="K5" s="72" t="str">
         <x:v>1</x:v>
@@ -1122,14 +1122,12 @@
       </x:c>
       <x:c r="N5" s="72" t="str"/>
       <x:c r="O5" s="72" t="str">
-        <x:v>STREEX-owned original — Juan</x:v>
+        <x:v>STREEX local fallback</x:v>
       </x:c>
       <x:c r="P5" s="72" t="str">
-        <x:v>User-owned original; permission confirmed</x:v>
-      </x:c>
-      <x:c r="Q5" s="72" t="str">
-        <x:v>Selected from IMG_3418.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
-      </x:c>
+        <x:v>No dedicated verified valley image currently active; the previously selected user photo was confirmed as Park City and was removed from activation.</x:v>
+      </x:c>
+      <x:c r="Q5" s="72" t="str"/>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="76" t="str">
@@ -1304,13 +1302,13 @@
         <x:v>Active in app</x:v>
       </x:c>
       <x:c r="G9" s="72" t="str">
-        <x:v>temple-square.jpg</x:v>
+        <x:v>temple-square-commons.jpg</x:v>
       </x:c>
       <x:c r="H9" s="72" t="str">
-        <x:v>/images/passenger/around-you/user/temple-square-spires-juan.webp</x:v>
+        <x:v>/images/passenger/around-you/temple-square.webp</x:v>
       </x:c>
       <x:c r="I9" s="74" t="str">
-        <x:v>Own local asset</x:v>
+        <x:v>Curated Commons asset</x:v>
       </x:c>
       <x:c r="J9" s="75" t="str">
         <x:v>No</x:v>
@@ -1324,15 +1322,17 @@
       <x:c r="M9" s="72" t="str">
         <x:v>Active coordinates</x:v>
       </x:c>
-      <x:c r="N9" s="72" t="str"/>
+      <x:c r="N9" s="72" t="str">
+        <x:v>https://commons.wikimedia.org/wiki/File:SLC_TempleSquare.jpg</x:v>
+      </x:c>
       <x:c r="O9" s="72" t="str">
-        <x:v>STREEX-owned original — Juan</x:v>
+        <x:v>Wikimedia Commons — Kenneth Hynek</x:v>
       </x:c>
       <x:c r="P9" s="72" t="str">
-        <x:v>User-owned original; permission confirmed</x:v>
+        <x:v>CC BY 2.0 — attribution required</x:v>
       </x:c>
       <x:c r="Q9" s="72" t="str">
-        <x:v>Selected from user-photos/temple-square-spires.jpeg; daylight hero showing Temple Square spires, architecture and grounds, optimized to local WebP with metadata stripped.</x:v>
+        <x:v>Dedicated Temple Square image downloaded, cropped and optimized locally. The legacy staged file was actually Kaysville Temple and was renamed to kaysville-temple.jpg.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
@@ -1358,13 +1358,13 @@
         <x:v>city-creek-canyon.jpg</x:v>
       </x:c>
       <x:c r="H10" s="76" t="str">
-        <x:v>/images/passenger/around-you/user/city-creek-canyon-juan.webp</x:v>
+        <x:v>/images/passenger/around-you/salt-lake-valley.webp</x:v>
       </x:c>
       <x:c r="I10" s="74" t="str">
-        <x:v>Own local asset</x:v>
+        <x:v>Shared fallback</x:v>
       </x:c>
       <x:c r="J10" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="K10" s="76" t="str">
         <x:v>1</x:v>
@@ -1377,14 +1377,12 @@
       </x:c>
       <x:c r="N10" s="76" t="str"/>
       <x:c r="O10" s="76" t="str">
-        <x:v>STREEX-owned original — Juan</x:v>
+        <x:v>STREEX local fallback</x:v>
       </x:c>
       <x:c r="P10" s="76" t="str">
-        <x:v>User-owned original; permission confirmed</x:v>
-      </x:c>
-      <x:c r="Q10" s="76" t="str">
-        <x:v>Selected from IMG_0976.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
-      </x:c>
+        <x:v>The supplied city-creek-canyon files were confirmed as Park City road and Capitol; a dedicated City Creek image is still required.</x:v>
+      </x:c>
+      <x:c r="Q10" s="76" t="str"/>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="72" t="str">
@@ -1927,10 +1925,10 @@
         <x:v>park-city.jpg</x:v>
       </x:c>
       <x:c r="H21" s="72" t="str">
-        <x:v>/images/passenger/around-you/user/park-city-juan.webp</x:v>
+        <x:v>/images/passenger/around-you/park-city.jpg</x:v>
       </x:c>
       <x:c r="I21" s="74" t="str">
-        <x:v>Own local asset</x:v>
+        <x:v>Curated local asset</x:v>
       </x:c>
       <x:c r="J21" s="75" t="str">
         <x:v>No</x:v>
@@ -1946,13 +1944,13 @@
       </x:c>
       <x:c r="N21" s="72" t="str"/>
       <x:c r="O21" s="72" t="str">
-        <x:v>STREEX-owned original — Juan</x:v>
+        <x:v>Existing app-local Park City image</x:v>
       </x:c>
       <x:c r="P21" s="72" t="str">
-        <x:v>User-owned original; permission confirmed</x:v>
+        <x:v>STREEX app asset</x:v>
       </x:c>
       <x:c r="Q21" s="72" t="str">
-        <x:v>Selected from IMG_4516.JPG; user-owned original optimized to local WebP with metadata stripped.</x:v>
+        <x:v>User park-city.JPG was deleted; corrected Park City road/valley originals remain in the source audit.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
@@ -1978,10 +1976,10 @@
         <x:v>historic-main-street.jpg</x:v>
       </x:c>
       <x:c r="H22" s="76" t="str">
-        <x:v>/images/passenger/around-you/user/historic-main-street-juan.webp</x:v>
+        <x:v>/images/passenger/around-you/historic-main-street.webp</x:v>
       </x:c>
       <x:c r="I22" s="74" t="str">
-        <x:v>Own local asset</x:v>
+        <x:v>Source local asset</x:v>
       </x:c>
       <x:c r="J22" s="75" t="str">
         <x:v>No</x:v>
@@ -1997,13 +1995,13 @@
       </x:c>
       <x:c r="N22" s="76" t="str"/>
       <x:c r="O22" s="76" t="str">
-        <x:v>STREEX-owned original — Juan</x:v>
+        <x:v>Existing app-local source asset</x:v>
       </x:c>
       <x:c r="P22" s="76" t="str">
-        <x:v>User-owned original; permission confirmed</x:v>
+        <x:v>STREEX app asset</x:v>
       </x:c>
       <x:c r="Q22" s="76" t="str">
-        <x:v>Selected from IMG_8782.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
+        <x:v>The active image is the existing Park City Main Street source asset; the user file historic-main-street.jpeg was confirmed as Downtown Salt Lake City and relabeled.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
@@ -2380,13 +2378,13 @@
         <x:v>the-gateway.jpg</x:v>
       </x:c>
       <x:c r="H30" s="76" t="str">
-        <x:v>/images/passenger/around-you/user/the-gateway-juan.webp</x:v>
+        <x:v>/images/passenger/around-you/downtown-slc.jpg</x:v>
       </x:c>
       <x:c r="I30" s="74" t="str">
-        <x:v>Own local asset</x:v>
+        <x:v>Shared fallback</x:v>
       </x:c>
       <x:c r="J30" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="K30" s="76" t="str">
         <x:v>1</x:v>
@@ -2399,14 +2397,12 @@
       </x:c>
       <x:c r="N30" s="76" t="str"/>
       <x:c r="O30" s="76" t="str">
-        <x:v>STREEX-owned original — Juan</x:v>
+        <x:v>STREEX local fallback</x:v>
       </x:c>
       <x:c r="P30" s="76" t="str">
-        <x:v>User-owned original; permission confirmed</x:v>
-      </x:c>
-      <x:c r="Q30" s="76" t="str">
-        <x:v>Selected from IMG_1412.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
-      </x:c>
+        <x:v>The supplied Gateway images were confirmed as Delta Center; a dedicated Gateway image is still required.</x:v>
+      </x:c>
+      <x:c r="Q30" s="76" t="str"/>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="72" t="str">
@@ -2480,13 +2476,13 @@
         <x:v>swaner-preserve.jpg</x:v>
       </x:c>
       <x:c r="H32" s="76" t="str">
-        <x:v>/images/passenger/around-you/user/swaner-preserve-juan.webp</x:v>
+        <x:v>/images/passenger/around-you/wasatch-back.webp</x:v>
       </x:c>
       <x:c r="I32" s="74" t="str">
-        <x:v>Own local asset</x:v>
+        <x:v>Shared fallback</x:v>
       </x:c>
       <x:c r="J32" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="K32" s="76" t="str">
         <x:v>1</x:v>
@@ -2499,14 +2495,12 @@
       </x:c>
       <x:c r="N32" s="76" t="str"/>
       <x:c r="O32" s="76" t="str">
-        <x:v>STREEX-owned original — Juan</x:v>
+        <x:v>STREEX local fallback</x:v>
       </x:c>
       <x:c r="P32" s="76" t="str">
-        <x:v>User-owned original; permission confirmed</x:v>
-      </x:c>
-      <x:c r="Q32" s="76" t="str">
-        <x:v>Selected from IMG_0264.jpeg; user-owned original optimized to local WebP with metadata stripped.</x:v>
-      </x:c>
+        <x:v>The supplied wetland photos were confirmed as Deer Valley; no Swaner-specific hero is activated.</x:v>
+      </x:c>
+      <x:c r="Q32" s="76" t="str"/>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="72" t="str">

</xml_diff>